<commit_message>
Update 0226084-SHDCO-LYM 1350 IO list.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/0226084-SHDCO-LYM 1350/0226084-SHDCO-LYM 1350 IO LIST.xlsx
+++ b/0226084-SHDCO-LYM 1350/0226084-SHDCO-LYM 1350 IO LIST.xlsx
@@ -4546,17 +4546,14 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="28" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -4572,43 +4569,17 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="37" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="37" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -4649,9 +4620,38 @@
     <xf numFmtId="0" fontId="20" fillId="11" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Köprü" xfId="1" builtinId="8"/>
@@ -11200,84 +11200,84 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="32.1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="92" t="s">
+      <c r="A1" s="116" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="92"/>
-      <c r="C1" s="92"/>
-      <c r="D1" s="92"/>
-      <c r="E1" s="92"/>
-      <c r="F1" s="92"/>
-      <c r="G1" s="92"/>
-      <c r="H1" s="92"/>
+      <c r="B1" s="116"/>
+      <c r="C1" s="116"/>
+      <c r="D1" s="116"/>
+      <c r="E1" s="116"/>
+      <c r="F1" s="116"/>
+      <c r="G1" s="116"/>
+      <c r="H1" s="116"/>
     </row>
     <row r="2" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="93" t="s">
+      <c r="A2" s="106" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="93"/>
-      <c r="C2" s="93"/>
-      <c r="D2" s="93"/>
-      <c r="E2" s="93"/>
-      <c r="F2" s="93"/>
-      <c r="G2" s="93"/>
-      <c r="H2" s="93"/>
+      <c r="B2" s="106"/>
+      <c r="C2" s="106"/>
+      <c r="D2" s="106"/>
+      <c r="E2" s="106"/>
+      <c r="F2" s="106"/>
+      <c r="G2" s="106"/>
+      <c r="H2" s="106"/>
     </row>
     <row r="4" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="90" t="s">
+      <c r="A4" s="114" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="90"/>
-      <c r="C4" s="90"/>
-      <c r="D4" s="90"/>
-      <c r="E4" s="90"/>
-      <c r="F4" s="90"/>
-      <c r="G4" s="90"/>
-      <c r="H4" s="90"/>
+      <c r="B4" s="114"/>
+      <c r="C4" s="114"/>
+      <c r="D4" s="114"/>
+      <c r="E4" s="114"/>
+      <c r="F4" s="114"/>
+      <c r="G4" s="114"/>
+      <c r="H4" s="114"/>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="85" t="s">
+      <c r="A5" s="84" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="85"/>
-      <c r="C5" s="85"/>
-      <c r="D5" s="85"/>
-      <c r="E5" s="85"/>
-      <c r="F5" s="85"/>
-      <c r="G5" s="85"/>
-      <c r="H5" s="85"/>
+      <c r="B5" s="84"/>
+      <c r="C5" s="84"/>
+      <c r="D5" s="84"/>
+      <c r="E5" s="84"/>
+      <c r="F5" s="84"/>
+      <c r="G5" s="84"/>
+      <c r="H5" s="84"/>
     </row>
     <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="85"/>
-      <c r="B6" s="85"/>
-      <c r="C6" s="85"/>
-      <c r="D6" s="85"/>
-      <c r="E6" s="85"/>
-      <c r="F6" s="85"/>
-      <c r="G6" s="85"/>
-      <c r="H6" s="85"/>
+      <c r="A6" s="84"/>
+      <c r="B6" s="84"/>
+      <c r="C6" s="84"/>
+      <c r="D6" s="84"/>
+      <c r="E6" s="84"/>
+      <c r="F6" s="84"/>
+      <c r="G6" s="84"/>
+      <c r="H6" s="84"/>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="85"/>
-      <c r="B7" s="85"/>
-      <c r="C7" s="85"/>
-      <c r="D7" s="85"/>
-      <c r="E7" s="85"/>
-      <c r="F7" s="85"/>
-      <c r="G7" s="85"/>
-      <c r="H7" s="85"/>
+      <c r="A7" s="84"/>
+      <c r="B7" s="84"/>
+      <c r="C7" s="84"/>
+      <c r="D7" s="84"/>
+      <c r="E7" s="84"/>
+      <c r="F7" s="84"/>
+      <c r="G7" s="84"/>
+      <c r="H7" s="84"/>
     </row>
     <row r="9" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="90" t="s">
+      <c r="A9" s="114" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="90"/>
-      <c r="C9" s="90"/>
-      <c r="D9" s="90"/>
-      <c r="E9" s="90"/>
-      <c r="F9" s="90"/>
-      <c r="G9" s="90"/>
-      <c r="H9" s="90"/>
+      <c r="B9" s="114"/>
+      <c r="C9" s="114"/>
+      <c r="D9" s="114"/>
+      <c r="E9" s="114"/>
+      <c r="F9" s="114"/>
+      <c r="G9" s="114"/>
+      <c r="H9" s="114"/>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
@@ -11436,16 +11436,16 @@
       </c>
     </row>
     <row r="16" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="90" t="s">
+      <c r="A16" s="114" t="s">
         <v>43</v>
       </c>
-      <c r="B16" s="90"/>
-      <c r="C16" s="90"/>
-      <c r="D16" s="90"/>
-      <c r="E16" s="90"/>
-      <c r="F16" s="90"/>
-      <c r="G16" s="90"/>
-      <c r="H16" s="90"/>
+      <c r="B16" s="114"/>
+      <c r="C16" s="114"/>
+      <c r="D16" s="114"/>
+      <c r="E16" s="114"/>
+      <c r="F16" s="114"/>
+      <c r="G16" s="114"/>
+      <c r="H16" s="114"/>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
@@ -11656,16 +11656,16 @@
       </c>
     </row>
     <row r="27" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="90" t="s">
+      <c r="A27" s="114" t="s">
         <v>74</v>
       </c>
-      <c r="B27" s="90"/>
-      <c r="C27" s="90"/>
-      <c r="D27" s="90"/>
-      <c r="E27" s="90"/>
-      <c r="F27" s="90"/>
-      <c r="G27" s="90"/>
-      <c r="H27" s="90"/>
+      <c r="B27" s="114"/>
+      <c r="C27" s="114"/>
+      <c r="D27" s="114"/>
+      <c r="E27" s="114"/>
+      <c r="F27" s="114"/>
+      <c r="G27" s="114"/>
+      <c r="H27" s="114"/>
     </row>
     <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
@@ -11931,16 +11931,16 @@
       <c r="E38" s="22"/>
     </row>
     <row r="39" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="90" t="s">
+      <c r="A39" s="114" t="s">
         <v>133</v>
       </c>
-      <c r="B39" s="90"/>
-      <c r="C39" s="90"/>
-      <c r="D39" s="90"/>
-      <c r="E39" s="91"/>
-      <c r="F39" s="90"/>
-      <c r="G39" s="90"/>
-      <c r="H39" s="90"/>
+      <c r="B39" s="114"/>
+      <c r="C39" s="114"/>
+      <c r="D39" s="114"/>
+      <c r="E39" s="115"/>
+      <c r="F39" s="114"/>
+      <c r="G39" s="114"/>
+      <c r="H39" s="114"/>
     </row>
     <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
@@ -12180,16 +12180,16 @@
       <c r="E49" s="22"/>
     </row>
     <row r="50" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="90" t="s">
+      <c r="A50" s="114" t="s">
         <v>194</v>
       </c>
-      <c r="B50" s="90"/>
-      <c r="C50" s="90"/>
-      <c r="D50" s="90"/>
-      <c r="E50" s="91"/>
-      <c r="F50" s="90"/>
-      <c r="G50" s="90"/>
-      <c r="H50" s="90"/>
+      <c r="B50" s="114"/>
+      <c r="C50" s="114"/>
+      <c r="D50" s="114"/>
+      <c r="E50" s="115"/>
+      <c r="F50" s="114"/>
+      <c r="G50" s="114"/>
+      <c r="H50" s="114"/>
     </row>
     <row r="51" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
@@ -12458,16 +12458,16 @@
       <c r="E62" s="22"/>
     </row>
     <row r="63" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="90" t="s">
+      <c r="A63" s="114" t="s">
         <v>255</v>
       </c>
-      <c r="B63" s="90"/>
-      <c r="C63" s="90"/>
-      <c r="D63" s="90"/>
-      <c r="E63" s="91"/>
-      <c r="F63" s="90"/>
-      <c r="G63" s="90"/>
-      <c r="H63" s="90"/>
+      <c r="B63" s="114"/>
+      <c r="C63" s="114"/>
+      <c r="D63" s="114"/>
+      <c r="E63" s="115"/>
+      <c r="F63" s="114"/>
+      <c r="G63" s="114"/>
+      <c r="H63" s="114"/>
     </row>
     <row r="64" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
@@ -12756,16 +12756,16 @@
       </c>
     </row>
     <row r="75" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="90" t="s">
+      <c r="A75" s="114" t="s">
         <v>313</v>
       </c>
-      <c r="B75" s="90"/>
-      <c r="C75" s="90"/>
-      <c r="D75" s="90"/>
-      <c r="E75" s="91"/>
-      <c r="F75" s="90"/>
-      <c r="G75" s="90"/>
-      <c r="H75" s="90"/>
+      <c r="B75" s="114"/>
+      <c r="C75" s="114"/>
+      <c r="D75" s="114"/>
+      <c r="E75" s="115"/>
+      <c r="F75" s="114"/>
+      <c r="G75" s="114"/>
+      <c r="H75" s="114"/>
     </row>
     <row r="76" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
@@ -13034,16 +13034,16 @@
       <c r="E87" s="22"/>
     </row>
     <row r="88" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="90" t="s">
+      <c r="A88" s="114" t="s">
         <v>390</v>
       </c>
-      <c r="B88" s="90"/>
-      <c r="C88" s="90"/>
-      <c r="D88" s="90"/>
-      <c r="E88" s="91"/>
-      <c r="F88" s="90"/>
-      <c r="G88" s="90"/>
-      <c r="H88" s="90"/>
+      <c r="B88" s="114"/>
+      <c r="C88" s="114"/>
+      <c r="D88" s="114"/>
+      <c r="E88" s="115"/>
+      <c r="F88" s="114"/>
+      <c r="G88" s="114"/>
+      <c r="H88" s="114"/>
     </row>
     <row r="89" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
@@ -13446,50 +13446,50 @@
       <c r="H104" s="25"/>
     </row>
     <row r="105" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="97" t="s">
+      <c r="A105" s="110" t="s">
         <v>475</v>
       </c>
-      <c r="B105" s="97"/>
-      <c r="C105" s="97"/>
-      <c r="D105" s="97"/>
-      <c r="E105" s="97"/>
-      <c r="F105" s="97"/>
-      <c r="G105" s="97"/>
-      <c r="H105" s="97"/>
+      <c r="B105" s="110"/>
+      <c r="C105" s="110"/>
+      <c r="D105" s="110"/>
+      <c r="E105" s="110"/>
+      <c r="F105" s="110"/>
+      <c r="G105" s="110"/>
+      <c r="H105" s="110"/>
     </row>
     <row r="107" spans="1:8" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A107" s="96" t="s">
+      <c r="A107" s="113" t="s">
         <v>476</v>
       </c>
-      <c r="B107" s="96"/>
-      <c r="C107" s="96"/>
-      <c r="D107" s="96"/>
-      <c r="E107" s="96"/>
-      <c r="F107" s="96"/>
-      <c r="G107" s="96"/>
-      <c r="H107" s="96"/>
+      <c r="B107" s="113"/>
+      <c r="C107" s="113"/>
+      <c r="D107" s="113"/>
+      <c r="E107" s="113"/>
+      <c r="F107" s="113"/>
+      <c r="G107" s="113"/>
+      <c r="H107" s="113"/>
     </row>
     <row r="108" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A108" s="97" t="s">
+      <c r="A108" s="110" t="s">
         <v>477</v>
       </c>
-      <c r="B108" s="97"/>
-      <c r="C108" s="97"/>
-      <c r="D108" s="97"/>
-      <c r="E108" s="97"/>
-      <c r="F108" s="97"/>
-      <c r="G108" s="97"/>
-      <c r="H108" s="97"/>
+      <c r="B108" s="110"/>
+      <c r="C108" s="110"/>
+      <c r="D108" s="110"/>
+      <c r="E108" s="110"/>
+      <c r="F108" s="110"/>
+      <c r="G108" s="110"/>
+      <c r="H108" s="110"/>
     </row>
     <row r="109" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="97"/>
-      <c r="B109" s="97"/>
-      <c r="C109" s="97"/>
-      <c r="D109" s="97"/>
-      <c r="E109" s="97"/>
-      <c r="F109" s="97"/>
-      <c r="G109" s="97"/>
-      <c r="H109" s="97"/>
+      <c r="A109" s="110"/>
+      <c r="B109" s="110"/>
+      <c r="C109" s="110"/>
+      <c r="D109" s="110"/>
+      <c r="E109" s="110"/>
+      <c r="F109" s="110"/>
+      <c r="G109" s="110"/>
+      <c r="H109" s="110"/>
     </row>
     <row r="111" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
@@ -14558,16 +14558,16 @@
       </c>
     </row>
     <row r="153" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A153" s="95" t="s">
+      <c r="A153" s="112" t="s">
         <v>663</v>
       </c>
-      <c r="B153" s="95"/>
-      <c r="C153" s="95"/>
-      <c r="D153" s="95"/>
-      <c r="E153" s="95"/>
-      <c r="F153" s="95"/>
-      <c r="G153" s="95"/>
-      <c r="H153" s="95"/>
+      <c r="B153" s="112"/>
+      <c r="C153" s="112"/>
+      <c r="D153" s="112"/>
+      <c r="E153" s="112"/>
+      <c r="F153" s="112"/>
+      <c r="G153" s="112"/>
+      <c r="H153" s="112"/>
     </row>
     <row r="154" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A154" s="35">
@@ -14576,14 +14576,14 @@
       <c r="B154" s="35" t="s">
         <v>664</v>
       </c>
-      <c r="C154" s="94" t="s">
+      <c r="C154" s="108" t="s">
         <v>665</v>
       </c>
-      <c r="D154" s="94"/>
-      <c r="E154" s="94"/>
-      <c r="F154" s="94"/>
-      <c r="G154" s="94"/>
-      <c r="H154" s="94"/>
+      <c r="D154" s="108"/>
+      <c r="E154" s="108"/>
+      <c r="F154" s="108"/>
+      <c r="G154" s="108"/>
+      <c r="H154" s="108"/>
     </row>
     <row r="155" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A155" s="35">
@@ -14592,14 +14592,14 @@
       <c r="B155" s="35" t="s">
         <v>666</v>
       </c>
-      <c r="C155" s="94" t="s">
+      <c r="C155" s="108" t="s">
         <v>667</v>
       </c>
-      <c r="D155" s="94"/>
-      <c r="E155" s="94"/>
-      <c r="F155" s="94"/>
-      <c r="G155" s="94"/>
-      <c r="H155" s="94"/>
+      <c r="D155" s="108"/>
+      <c r="E155" s="108"/>
+      <c r="F155" s="108"/>
+      <c r="G155" s="108"/>
+      <c r="H155" s="108"/>
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A156" s="35">
@@ -14608,14 +14608,14 @@
       <c r="B156" s="35" t="s">
         <v>668</v>
       </c>
-      <c r="C156" s="94" t="s">
+      <c r="C156" s="108" t="s">
         <v>669</v>
       </c>
-      <c r="D156" s="94"/>
-      <c r="E156" s="94"/>
-      <c r="F156" s="94"/>
-      <c r="G156" s="94"/>
-      <c r="H156" s="94"/>
+      <c r="D156" s="108"/>
+      <c r="E156" s="108"/>
+      <c r="F156" s="108"/>
+      <c r="G156" s="108"/>
+      <c r="H156" s="108"/>
     </row>
     <row r="157" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A157" s="35">
@@ -14624,14 +14624,14 @@
       <c r="B157" s="35" t="s">
         <v>570</v>
       </c>
-      <c r="C157" s="94" t="s">
+      <c r="C157" s="108" t="s">
         <v>670</v>
       </c>
-      <c r="D157" s="94"/>
-      <c r="E157" s="94"/>
-      <c r="F157" s="94"/>
-      <c r="G157" s="94"/>
-      <c r="H157" s="94"/>
+      <c r="D157" s="108"/>
+      <c r="E157" s="108"/>
+      <c r="F157" s="108"/>
+      <c r="G157" s="108"/>
+      <c r="H157" s="108"/>
     </row>
     <row r="158" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A158" s="35">
@@ -14640,14 +14640,14 @@
       <c r="B158" s="35" t="s">
         <v>671</v>
       </c>
-      <c r="C158" s="94" t="s">
+      <c r="C158" s="108" t="s">
         <v>672</v>
       </c>
-      <c r="D158" s="94"/>
-      <c r="E158" s="94"/>
-      <c r="F158" s="94"/>
-      <c r="G158" s="94"/>
-      <c r="H158" s="94"/>
+      <c r="D158" s="108"/>
+      <c r="E158" s="108"/>
+      <c r="F158" s="108"/>
+      <c r="G158" s="108"/>
+      <c r="H158" s="108"/>
     </row>
     <row r="159" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A159" s="35">
@@ -14656,26 +14656,26 @@
       <c r="B159" s="35" t="s">
         <v>673</v>
       </c>
-      <c r="C159" s="94" t="s">
+      <c r="C159" s="108" t="s">
         <v>674</v>
       </c>
-      <c r="D159" s="94"/>
-      <c r="E159" s="94"/>
-      <c r="F159" s="94"/>
-      <c r="G159" s="94"/>
-      <c r="H159" s="94"/>
+      <c r="D159" s="108"/>
+      <c r="E159" s="108"/>
+      <c r="F159" s="108"/>
+      <c r="G159" s="108"/>
+      <c r="H159" s="108"/>
     </row>
     <row r="161" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A161" s="95" t="s">
+      <c r="A161" s="112" t="s">
         <v>675</v>
       </c>
-      <c r="B161" s="95"/>
-      <c r="C161" s="95"/>
-      <c r="D161" s="95"/>
-      <c r="E161" s="95"/>
-      <c r="F161" s="95"/>
-      <c r="G161" s="95"/>
-      <c r="H161" s="95"/>
+      <c r="B161" s="112"/>
+      <c r="C161" s="112"/>
+      <c r="D161" s="112"/>
+      <c r="E161" s="112"/>
+      <c r="F161" s="112"/>
+      <c r="G161" s="112"/>
+      <c r="H161" s="112"/>
     </row>
     <row r="162" spans="1:8" ht="48.75" x14ac:dyDescent="0.25">
       <c r="A162" s="36" t="s">
@@ -14848,48 +14848,48 @@
       <c r="H170" s="36"/>
     </row>
     <row r="172" spans="1:8" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A172" s="96" t="s">
+      <c r="A172" s="113" t="s">
         <v>713</v>
       </c>
-      <c r="B172" s="96"/>
-      <c r="C172" s="96"/>
-      <c r="D172" s="96"/>
-      <c r="E172" s="96"/>
-      <c r="F172" s="96"/>
-      <c r="G172" s="96"/>
-      <c r="H172" s="96"/>
+      <c r="B172" s="113"/>
+      <c r="C172" s="113"/>
+      <c r="D172" s="113"/>
+      <c r="E172" s="113"/>
+      <c r="F172" s="113"/>
+      <c r="G172" s="113"/>
+      <c r="H172" s="113"/>
     </row>
     <row r="173" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A173" s="97" t="s">
+      <c r="A173" s="110" t="s">
         <v>714</v>
       </c>
-      <c r="B173" s="97"/>
-      <c r="C173" s="97"/>
-      <c r="D173" s="97"/>
-      <c r="E173" s="97"/>
-      <c r="F173" s="97"/>
-      <c r="G173" s="97"/>
-      <c r="H173" s="97"/>
+      <c r="B173" s="110"/>
+      <c r="C173" s="110"/>
+      <c r="D173" s="110"/>
+      <c r="E173" s="110"/>
+      <c r="F173" s="110"/>
+      <c r="G173" s="110"/>
+      <c r="H173" s="110"/>
     </row>
     <row r="174" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A174" s="97"/>
-      <c r="B174" s="97"/>
-      <c r="C174" s="97"/>
-      <c r="D174" s="97"/>
-      <c r="E174" s="97"/>
-      <c r="F174" s="97"/>
-      <c r="G174" s="97"/>
-      <c r="H174" s="97"/>
+      <c r="A174" s="110"/>
+      <c r="B174" s="110"/>
+      <c r="C174" s="110"/>
+      <c r="D174" s="110"/>
+      <c r="E174" s="110"/>
+      <c r="F174" s="110"/>
+      <c r="G174" s="110"/>
+      <c r="H174" s="110"/>
     </row>
     <row r="175" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A175" s="97"/>
-      <c r="B175" s="97"/>
-      <c r="C175" s="97"/>
-      <c r="D175" s="97"/>
-      <c r="E175" s="97"/>
-      <c r="F175" s="97"/>
-      <c r="G175" s="97"/>
-      <c r="H175" s="97"/>
+      <c r="A175" s="110"/>
+      <c r="B175" s="110"/>
+      <c r="C175" s="110"/>
+      <c r="D175" s="110"/>
+      <c r="E175" s="110"/>
+      <c r="F175" s="110"/>
+      <c r="G175" s="110"/>
+      <c r="H175" s="110"/>
     </row>
     <row r="177" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
@@ -15100,16 +15100,16 @@
       </c>
     </row>
     <row r="186" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A186" s="95" t="s">
+      <c r="A186" s="112" t="s">
         <v>772</v>
       </c>
-      <c r="B186" s="95"/>
-      <c r="C186" s="95"/>
-      <c r="D186" s="95"/>
-      <c r="E186" s="95"/>
-      <c r="F186" s="95"/>
-      <c r="G186" s="95"/>
-      <c r="H186" s="95"/>
+      <c r="B186" s="112"/>
+      <c r="C186" s="112"/>
+      <c r="D186" s="112"/>
+      <c r="E186" s="112"/>
+      <c r="F186" s="112"/>
+      <c r="G186" s="112"/>
+      <c r="H186" s="112"/>
     </row>
     <row r="187" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A187" s="35">
@@ -15121,13 +15121,13 @@
       <c r="C187" s="35" t="s">
         <v>774</v>
       </c>
-      <c r="D187" s="94" t="s">
+      <c r="D187" s="108" t="s">
         <v>775</v>
       </c>
-      <c r="E187" s="94"/>
-      <c r="F187" s="94"/>
-      <c r="G187" s="94"/>
-      <c r="H187" s="94"/>
+      <c r="E187" s="108"/>
+      <c r="F187" s="108"/>
+      <c r="G187" s="108"/>
+      <c r="H187" s="108"/>
     </row>
     <row r="188" spans="1:8" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A188" s="35">
@@ -15139,13 +15139,13 @@
       <c r="C188" s="35" t="s">
         <v>777</v>
       </c>
-      <c r="D188" s="94" t="s">
+      <c r="D188" s="108" t="s">
         <v>778</v>
       </c>
-      <c r="E188" s="94"/>
-      <c r="F188" s="94"/>
-      <c r="G188" s="94"/>
-      <c r="H188" s="94"/>
+      <c r="E188" s="108"/>
+      <c r="F188" s="108"/>
+      <c r="G188" s="108"/>
+      <c r="H188" s="108"/>
     </row>
     <row r="189" spans="1:8" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A189" s="35">
@@ -15157,13 +15157,13 @@
       <c r="C189" s="35" t="s">
         <v>780</v>
       </c>
-      <c r="D189" s="94" t="s">
+      <c r="D189" s="108" t="s">
         <v>781</v>
       </c>
-      <c r="E189" s="94"/>
-      <c r="F189" s="94"/>
-      <c r="G189" s="94"/>
-      <c r="H189" s="94"/>
+      <c r="E189" s="108"/>
+      <c r="F189" s="108"/>
+      <c r="G189" s="108"/>
+      <c r="H189" s="108"/>
     </row>
     <row r="190" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A190" s="35">
@@ -15175,13 +15175,13 @@
       <c r="C190" s="35" t="s">
         <v>783</v>
       </c>
-      <c r="D190" s="94" t="s">
+      <c r="D190" s="108" t="s">
         <v>784</v>
       </c>
-      <c r="E190" s="94"/>
-      <c r="F190" s="94"/>
-      <c r="G190" s="94"/>
-      <c r="H190" s="94"/>
+      <c r="E190" s="108"/>
+      <c r="F190" s="108"/>
+      <c r="G190" s="108"/>
+      <c r="H190" s="108"/>
     </row>
     <row r="191" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A191" s="35">
@@ -15193,37 +15193,37 @@
       <c r="C191" s="35" t="s">
         <v>786</v>
       </c>
-      <c r="D191" s="94" t="s">
+      <c r="D191" s="108" t="s">
         <v>787</v>
       </c>
-      <c r="E191" s="94"/>
-      <c r="F191" s="94"/>
-      <c r="G191" s="94"/>
-      <c r="H191" s="94"/>
+      <c r="E191" s="108"/>
+      <c r="F191" s="108"/>
+      <c r="G191" s="108"/>
+      <c r="H191" s="108"/>
     </row>
     <row r="193" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A193" s="98" t="s">
+      <c r="A193" s="109" t="s">
         <v>788</v>
       </c>
-      <c r="B193" s="98"/>
-      <c r="C193" s="98"/>
-      <c r="D193" s="98"/>
-      <c r="E193" s="98"/>
-      <c r="F193" s="98"/>
-      <c r="G193" s="98"/>
-      <c r="H193" s="98"/>
+      <c r="B193" s="109"/>
+      <c r="C193" s="109"/>
+      <c r="D193" s="109"/>
+      <c r="E193" s="109"/>
+      <c r="F193" s="109"/>
+      <c r="G193" s="109"/>
+      <c r="H193" s="109"/>
     </row>
     <row r="194" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A194" s="93" t="s">
+      <c r="A194" s="106" t="s">
         <v>789</v>
       </c>
-      <c r="B194" s="93"/>
-      <c r="C194" s="93"/>
-      <c r="D194" s="93"/>
-      <c r="E194" s="93"/>
-      <c r="F194" s="93"/>
-      <c r="G194" s="93"/>
-      <c r="H194" s="93"/>
+      <c r="B194" s="106"/>
+      <c r="C194" s="106"/>
+      <c r="D194" s="106"/>
+      <c r="E194" s="106"/>
+      <c r="F194" s="106"/>
+      <c r="G194" s="106"/>
+      <c r="H194" s="106"/>
     </row>
     <row r="196" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="197" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -15284,968 +15284,968 @@
     <row r="252" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="253" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="254" spans="1:8" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A254" s="97" t="s">
+      <c r="A254" s="110" t="s">
         <v>790</v>
       </c>
-      <c r="B254" s="97"/>
-      <c r="C254" s="97"/>
-      <c r="D254" s="97"/>
-      <c r="E254" s="97"/>
-      <c r="F254" s="97"/>
-      <c r="G254" s="97"/>
-      <c r="H254" s="97"/>
+      <c r="B254" s="110"/>
+      <c r="C254" s="110"/>
+      <c r="D254" s="110"/>
+      <c r="E254" s="110"/>
+      <c r="F254" s="110"/>
+      <c r="G254" s="110"/>
+      <c r="H254" s="110"/>
     </row>
     <row r="255" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A255" s="99" t="s">
+      <c r="A255" s="111" t="s">
         <v>791</v>
       </c>
-      <c r="B255" s="99"/>
-      <c r="C255" s="99"/>
-      <c r="D255" s="99"/>
-      <c r="E255" s="99"/>
-      <c r="F255" s="99"/>
-      <c r="G255" s="99"/>
-      <c r="H255" s="99"/>
+      <c r="B255" s="111"/>
+      <c r="C255" s="111"/>
+      <c r="D255" s="111"/>
+      <c r="E255" s="111"/>
+      <c r="F255" s="111"/>
+      <c r="G255" s="111"/>
+      <c r="H255" s="111"/>
     </row>
     <row r="257" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A257" s="98" t="s">
+      <c r="A257" s="109" t="s">
         <v>792</v>
       </c>
-      <c r="B257" s="98"/>
-      <c r="C257" s="98"/>
-      <c r="D257" s="98"/>
-      <c r="E257" s="98"/>
-      <c r="F257" s="98"/>
-      <c r="G257" s="98"/>
-      <c r="H257" s="98"/>
+      <c r="B257" s="109"/>
+      <c r="C257" s="109"/>
+      <c r="D257" s="109"/>
+      <c r="E257" s="109"/>
+      <c r="F257" s="109"/>
+      <c r="G257" s="109"/>
+      <c r="H257" s="109"/>
     </row>
     <row r="258" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A258" s="93" t="s">
+      <c r="A258" s="106" t="s">
         <v>793</v>
       </c>
-      <c r="B258" s="93"/>
-      <c r="C258" s="93"/>
-      <c r="D258" s="93"/>
-      <c r="E258" s="93"/>
-      <c r="F258" s="93"/>
-      <c r="G258" s="93"/>
-      <c r="H258" s="93"/>
+      <c r="B258" s="106"/>
+      <c r="C258" s="106"/>
+      <c r="D258" s="106"/>
+      <c r="E258" s="106"/>
+      <c r="F258" s="106"/>
+      <c r="G258" s="106"/>
+      <c r="H258" s="106"/>
     </row>
     <row r="260" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A260" s="102" t="s">
+      <c r="A260" s="107" t="s">
         <v>794</v>
       </c>
-      <c r="B260" s="102"/>
-      <c r="C260" s="102"/>
-      <c r="D260" s="102"/>
-      <c r="E260" s="102" t="s">
+      <c r="B260" s="107"/>
+      <c r="C260" s="107"/>
+      <c r="D260" s="107"/>
+      <c r="E260" s="107" t="s">
         <v>795</v>
       </c>
-      <c r="F260" s="102"/>
-      <c r="G260" s="102"/>
-      <c r="H260" s="102"/>
+      <c r="F260" s="107"/>
+      <c r="G260" s="107"/>
+      <c r="H260" s="107"/>
     </row>
     <row r="261" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A261" s="100" t="s">
+      <c r="A261" s="104" t="s">
         <v>796</v>
       </c>
-      <c r="B261" s="100"/>
-      <c r="C261" s="100"/>
-      <c r="D261" s="100"/>
-      <c r="E261" s="100" t="s">
+      <c r="B261" s="104"/>
+      <c r="C261" s="104"/>
+      <c r="D261" s="104"/>
+      <c r="E261" s="104" t="s">
         <v>797</v>
       </c>
-      <c r="F261" s="100"/>
-      <c r="G261" s="100"/>
-      <c r="H261" s="100"/>
+      <c r="F261" s="104"/>
+      <c r="G261" s="104"/>
+      <c r="H261" s="104"/>
     </row>
     <row r="262" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A262" s="101" t="s">
+      <c r="A262" s="103" t="s">
         <v>798</v>
       </c>
-      <c r="B262" s="101"/>
-      <c r="C262" s="101"/>
-      <c r="D262" s="101"/>
-      <c r="E262" s="101" t="s">
+      <c r="B262" s="103"/>
+      <c r="C262" s="103"/>
+      <c r="D262" s="103"/>
+      <c r="E262" s="103" t="s">
         <v>799</v>
       </c>
-      <c r="F262" s="101"/>
-      <c r="G262" s="101"/>
-      <c r="H262" s="101"/>
+      <c r="F262" s="103"/>
+      <c r="G262" s="103"/>
+      <c r="H262" s="103"/>
     </row>
     <row r="263" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A263" s="100" t="s">
+      <c r="A263" s="104" t="s">
         <v>494</v>
       </c>
-      <c r="B263" s="100"/>
-      <c r="C263" s="100"/>
-      <c r="D263" s="100"/>
-      <c r="E263" s="100" t="s">
+      <c r="B263" s="104"/>
+      <c r="C263" s="104"/>
+      <c r="D263" s="104"/>
+      <c r="E263" s="104" t="s">
         <v>800</v>
       </c>
-      <c r="F263" s="100"/>
-      <c r="G263" s="100"/>
-      <c r="H263" s="100"/>
+      <c r="F263" s="104"/>
+      <c r="G263" s="104"/>
+      <c r="H263" s="104"/>
     </row>
     <row r="264" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A264" s="101" t="s">
+      <c r="A264" s="103" t="s">
         <v>801</v>
       </c>
-      <c r="B264" s="101"/>
-      <c r="C264" s="101"/>
-      <c r="D264" s="101"/>
-      <c r="E264" s="101" t="s">
+      <c r="B264" s="103"/>
+      <c r="C264" s="103"/>
+      <c r="D264" s="103"/>
+      <c r="E264" s="103" t="s">
         <v>802</v>
       </c>
-      <c r="F264" s="101"/>
-      <c r="G264" s="101"/>
-      <c r="H264" s="101"/>
+      <c r="F264" s="103"/>
+      <c r="G264" s="103"/>
+      <c r="H264" s="103"/>
     </row>
     <row r="265" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A265" s="100" t="s">
+      <c r="A265" s="104" t="s">
         <v>503</v>
       </c>
-      <c r="B265" s="100"/>
-      <c r="C265" s="100"/>
-      <c r="D265" s="100"/>
-      <c r="E265" s="100" t="s">
+      <c r="B265" s="104"/>
+      <c r="C265" s="104"/>
+      <c r="D265" s="104"/>
+      <c r="E265" s="104" t="s">
         <v>803</v>
       </c>
-      <c r="F265" s="100"/>
-      <c r="G265" s="100"/>
-      <c r="H265" s="100"/>
+      <c r="F265" s="104"/>
+      <c r="G265" s="104"/>
+      <c r="H265" s="104"/>
     </row>
     <row r="266" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A266" s="101" t="s">
+      <c r="A266" s="103" t="s">
         <v>553</v>
       </c>
-      <c r="B266" s="101"/>
-      <c r="C266" s="101"/>
-      <c r="D266" s="101"/>
-      <c r="E266" s="101" t="s">
+      <c r="B266" s="103"/>
+      <c r="C266" s="103"/>
+      <c r="D266" s="103"/>
+      <c r="E266" s="103" t="s">
         <v>804</v>
       </c>
-      <c r="F266" s="101"/>
-      <c r="G266" s="101"/>
-      <c r="H266" s="101"/>
+      <c r="F266" s="103"/>
+      <c r="G266" s="103"/>
+      <c r="H266" s="103"/>
     </row>
     <row r="267" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A267" s="100" t="s">
+      <c r="A267" s="104" t="s">
         <v>805</v>
       </c>
-      <c r="B267" s="100"/>
-      <c r="C267" s="100"/>
-      <c r="D267" s="100"/>
-      <c r="E267" s="100" t="s">
+      <c r="B267" s="104"/>
+      <c r="C267" s="104"/>
+      <c r="D267" s="104"/>
+      <c r="E267" s="104" t="s">
         <v>806</v>
       </c>
-      <c r="F267" s="100"/>
-      <c r="G267" s="100"/>
-      <c r="H267" s="100"/>
+      <c r="F267" s="104"/>
+      <c r="G267" s="104"/>
+      <c r="H267" s="104"/>
     </row>
     <row r="268" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A268" s="101" t="s">
+      <c r="A268" s="103" t="s">
         <v>512</v>
       </c>
-      <c r="B268" s="101"/>
-      <c r="C268" s="101"/>
-      <c r="D268" s="101"/>
-      <c r="E268" s="101" t="s">
+      <c r="B268" s="103"/>
+      <c r="C268" s="103"/>
+      <c r="D268" s="103"/>
+      <c r="E268" s="103" t="s">
         <v>807</v>
       </c>
-      <c r="F268" s="101"/>
-      <c r="G268" s="101"/>
-      <c r="H268" s="101"/>
+      <c r="F268" s="103"/>
+      <c r="G268" s="103"/>
+      <c r="H268" s="103"/>
     </row>
     <row r="269" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A269" s="100" t="s">
+      <c r="A269" s="104" t="s">
         <v>516</v>
       </c>
-      <c r="B269" s="100"/>
-      <c r="C269" s="100"/>
-      <c r="D269" s="100"/>
-      <c r="E269" s="100" t="s">
+      <c r="B269" s="104"/>
+      <c r="C269" s="104"/>
+      <c r="D269" s="104"/>
+      <c r="E269" s="104" t="s">
         <v>808</v>
       </c>
-      <c r="F269" s="100"/>
-      <c r="G269" s="100"/>
-      <c r="H269" s="100"/>
+      <c r="F269" s="104"/>
+      <c r="G269" s="104"/>
+      <c r="H269" s="104"/>
     </row>
     <row r="270" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A270" s="101" t="s">
+      <c r="A270" s="103" t="s">
         <v>704</v>
       </c>
-      <c r="B270" s="101"/>
-      <c r="C270" s="101"/>
-      <c r="D270" s="101"/>
-      <c r="E270" s="101" t="s">
+      <c r="B270" s="103"/>
+      <c r="C270" s="103"/>
+      <c r="D270" s="103"/>
+      <c r="E270" s="103" t="s">
         <v>809</v>
       </c>
-      <c r="F270" s="101"/>
-      <c r="G270" s="101"/>
-      <c r="H270" s="101"/>
+      <c r="F270" s="103"/>
+      <c r="G270" s="103"/>
+      <c r="H270" s="103"/>
     </row>
     <row r="271" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A271" s="100" t="s">
+      <c r="A271" s="104" t="s">
         <v>683</v>
       </c>
-      <c r="B271" s="100"/>
-      <c r="C271" s="100"/>
-      <c r="D271" s="100"/>
-      <c r="E271" s="100" t="s">
+      <c r="B271" s="104"/>
+      <c r="C271" s="104"/>
+      <c r="D271" s="104"/>
+      <c r="E271" s="104" t="s">
         <v>810</v>
       </c>
-      <c r="F271" s="100"/>
-      <c r="G271" s="100"/>
-      <c r="H271" s="100"/>
+      <c r="F271" s="104"/>
+      <c r="G271" s="104"/>
+      <c r="H271" s="104"/>
     </row>
     <row r="272" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A272" s="101" t="s">
+      <c r="A272" s="103" t="s">
         <v>811</v>
       </c>
-      <c r="B272" s="101"/>
-      <c r="C272" s="101"/>
-      <c r="D272" s="101"/>
-      <c r="E272" s="101" t="s">
+      <c r="B272" s="103"/>
+      <c r="C272" s="103"/>
+      <c r="D272" s="103"/>
+      <c r="E272" s="103" t="s">
         <v>812</v>
       </c>
-      <c r="F272" s="101"/>
-      <c r="G272" s="101"/>
-      <c r="H272" s="101"/>
+      <c r="F272" s="103"/>
+      <c r="G272" s="103"/>
+      <c r="H272" s="103"/>
     </row>
     <row r="273" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A273" s="100" t="s">
+      <c r="A273" s="104" t="s">
         <v>813</v>
       </c>
-      <c r="B273" s="100"/>
-      <c r="C273" s="100"/>
-      <c r="D273" s="100"/>
-      <c r="E273" s="100" t="s">
+      <c r="B273" s="104"/>
+      <c r="C273" s="104"/>
+      <c r="D273" s="104"/>
+      <c r="E273" s="104" t="s">
         <v>814</v>
       </c>
-      <c r="F273" s="100"/>
-      <c r="G273" s="100"/>
-      <c r="H273" s="100"/>
+      <c r="F273" s="104"/>
+      <c r="G273" s="104"/>
+      <c r="H273" s="104"/>
     </row>
     <row r="274" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A274" s="101" t="s">
+      <c r="A274" s="103" t="s">
         <v>815</v>
       </c>
-      <c r="B274" s="101"/>
-      <c r="C274" s="101"/>
-      <c r="D274" s="101"/>
-      <c r="E274" s="101" t="s">
+      <c r="B274" s="103"/>
+      <c r="C274" s="103"/>
+      <c r="D274" s="103"/>
+      <c r="E274" s="103" t="s">
         <v>816</v>
       </c>
-      <c r="F274" s="101"/>
-      <c r="G274" s="101"/>
-      <c r="H274" s="101"/>
+      <c r="F274" s="103"/>
+      <c r="G274" s="103"/>
+      <c r="H274" s="103"/>
     </row>
     <row r="275" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A275" s="100" t="s">
+      <c r="A275" s="104" t="s">
         <v>817</v>
       </c>
-      <c r="B275" s="100"/>
-      <c r="C275" s="100"/>
-      <c r="D275" s="100"/>
-      <c r="E275" s="100" t="s">
+      <c r="B275" s="104"/>
+      <c r="C275" s="104"/>
+      <c r="D275" s="104"/>
+      <c r="E275" s="104" t="s">
         <v>818</v>
       </c>
-      <c r="F275" s="100"/>
-      <c r="G275" s="100"/>
-      <c r="H275" s="100"/>
+      <c r="F275" s="104"/>
+      <c r="G275" s="104"/>
+      <c r="H275" s="104"/>
     </row>
     <row r="276" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A276" s="101" t="s">
+      <c r="A276" s="103" t="s">
         <v>819</v>
       </c>
-      <c r="B276" s="101"/>
-      <c r="C276" s="101"/>
-      <c r="D276" s="101"/>
-      <c r="E276" s="101" t="s">
+      <c r="B276" s="103"/>
+      <c r="C276" s="103"/>
+      <c r="D276" s="103"/>
+      <c r="E276" s="103" t="s">
         <v>820</v>
       </c>
-      <c r="F276" s="101"/>
-      <c r="G276" s="101"/>
-      <c r="H276" s="101"/>
+      <c r="F276" s="103"/>
+      <c r="G276" s="103"/>
+      <c r="H276" s="103"/>
     </row>
     <row r="277" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A277" s="100" t="s">
+      <c r="A277" s="104" t="s">
         <v>821</v>
       </c>
-      <c r="B277" s="100"/>
-      <c r="C277" s="100"/>
-      <c r="D277" s="100"/>
-      <c r="E277" s="100" t="s">
+      <c r="B277" s="104"/>
+      <c r="C277" s="104"/>
+      <c r="D277" s="104"/>
+      <c r="E277" s="104" t="s">
         <v>822</v>
       </c>
-      <c r="F277" s="100"/>
-      <c r="G277" s="100"/>
-      <c r="H277" s="100"/>
+      <c r="F277" s="104"/>
+      <c r="G277" s="104"/>
+      <c r="H277" s="104"/>
     </row>
     <row r="278" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A278" s="101" t="s">
+      <c r="A278" s="103" t="s">
         <v>823</v>
       </c>
-      <c r="B278" s="101"/>
-      <c r="C278" s="101"/>
-      <c r="D278" s="101"/>
-      <c r="E278" s="101" t="s">
+      <c r="B278" s="103"/>
+      <c r="C278" s="103"/>
+      <c r="D278" s="103"/>
+      <c r="E278" s="103" t="s">
         <v>824</v>
       </c>
-      <c r="F278" s="101"/>
-      <c r="G278" s="101"/>
-      <c r="H278" s="101"/>
+      <c r="F278" s="103"/>
+      <c r="G278" s="103"/>
+      <c r="H278" s="103"/>
     </row>
     <row r="279" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A279" s="100" t="s">
+      <c r="A279" s="104" t="s">
         <v>825</v>
       </c>
-      <c r="B279" s="100"/>
-      <c r="C279" s="100"/>
-      <c r="D279" s="100"/>
-      <c r="E279" s="100" t="s">
+      <c r="B279" s="104"/>
+      <c r="C279" s="104"/>
+      <c r="D279" s="104"/>
+      <c r="E279" s="104" t="s">
         <v>826</v>
       </c>
-      <c r="F279" s="100"/>
-      <c r="G279" s="100"/>
-      <c r="H279" s="100"/>
+      <c r="F279" s="104"/>
+      <c r="G279" s="104"/>
+      <c r="H279" s="104"/>
     </row>
     <row r="280" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A280" s="101" t="s">
+      <c r="A280" s="103" t="s">
         <v>827</v>
       </c>
-      <c r="B280" s="101"/>
-      <c r="C280" s="101"/>
-      <c r="D280" s="101"/>
-      <c r="E280" s="101" t="s">
+      <c r="B280" s="103"/>
+      <c r="C280" s="103"/>
+      <c r="D280" s="103"/>
+      <c r="E280" s="103" t="s">
         <v>828</v>
       </c>
-      <c r="F280" s="101"/>
-      <c r="G280" s="101"/>
-      <c r="H280" s="101"/>
+      <c r="F280" s="103"/>
+      <c r="G280" s="103"/>
+      <c r="H280" s="103"/>
     </row>
     <row r="281" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A281" s="100" t="s">
+      <c r="A281" s="104" t="s">
         <v>829</v>
       </c>
-      <c r="B281" s="100"/>
-      <c r="C281" s="100"/>
-      <c r="D281" s="100"/>
-      <c r="E281" s="100" t="s">
+      <c r="B281" s="104"/>
+      <c r="C281" s="104"/>
+      <c r="D281" s="104"/>
+      <c r="E281" s="104" t="s">
         <v>830</v>
       </c>
-      <c r="F281" s="100"/>
-      <c r="G281" s="100"/>
-      <c r="H281" s="100"/>
+      <c r="F281" s="104"/>
+      <c r="G281" s="104"/>
+      <c r="H281" s="104"/>
     </row>
     <row r="282" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A282" s="101" t="s">
+      <c r="A282" s="103" t="s">
         <v>831</v>
       </c>
-      <c r="B282" s="101"/>
-      <c r="C282" s="101"/>
-      <c r="D282" s="101"/>
-      <c r="E282" s="101" t="s">
+      <c r="B282" s="103"/>
+      <c r="C282" s="103"/>
+      <c r="D282" s="103"/>
+      <c r="E282" s="103" t="s">
         <v>832</v>
       </c>
-      <c r="F282" s="101"/>
-      <c r="G282" s="101"/>
-      <c r="H282" s="101"/>
+      <c r="F282" s="103"/>
+      <c r="G282" s="103"/>
+      <c r="H282" s="103"/>
     </row>
     <row r="283" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A283" s="100" t="s">
+      <c r="A283" s="104" t="s">
         <v>833</v>
       </c>
-      <c r="B283" s="100"/>
-      <c r="C283" s="100"/>
-      <c r="D283" s="100"/>
-      <c r="E283" s="100" t="s">
+      <c r="B283" s="104"/>
+      <c r="C283" s="104"/>
+      <c r="D283" s="104"/>
+      <c r="E283" s="104" t="s">
         <v>834</v>
       </c>
-      <c r="F283" s="100"/>
-      <c r="G283" s="100"/>
-      <c r="H283" s="100"/>
+      <c r="F283" s="104"/>
+      <c r="G283" s="104"/>
+      <c r="H283" s="104"/>
     </row>
     <row r="284" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A284" s="101" t="s">
+      <c r="A284" s="103" t="s">
         <v>835</v>
       </c>
-      <c r="B284" s="101"/>
-      <c r="C284" s="101"/>
-      <c r="D284" s="101"/>
-      <c r="E284" s="101" t="s">
+      <c r="B284" s="103"/>
+      <c r="C284" s="103"/>
+      <c r="D284" s="103"/>
+      <c r="E284" s="103" t="s">
         <v>836</v>
       </c>
-      <c r="F284" s="101"/>
-      <c r="G284" s="101"/>
-      <c r="H284" s="101"/>
+      <c r="F284" s="103"/>
+      <c r="G284" s="103"/>
+      <c r="H284" s="103"/>
     </row>
     <row r="285" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A285" s="100" t="s">
+      <c r="A285" s="104" t="s">
         <v>837</v>
       </c>
-      <c r="B285" s="100"/>
-      <c r="C285" s="100"/>
-      <c r="D285" s="100"/>
-      <c r="E285" s="100" t="s">
+      <c r="B285" s="104"/>
+      <c r="C285" s="104"/>
+      <c r="D285" s="104"/>
+      <c r="E285" s="104" t="s">
         <v>838</v>
       </c>
-      <c r="F285" s="100"/>
-      <c r="G285" s="100"/>
-      <c r="H285" s="100"/>
+      <c r="F285" s="104"/>
+      <c r="G285" s="104"/>
+      <c r="H285" s="104"/>
     </row>
     <row r="286" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A286" s="101" t="s">
+      <c r="A286" s="103" t="s">
         <v>839</v>
       </c>
-      <c r="B286" s="101"/>
-      <c r="C286" s="101"/>
-      <c r="D286" s="101"/>
-      <c r="E286" s="101" t="s">
+      <c r="B286" s="103"/>
+      <c r="C286" s="103"/>
+      <c r="D286" s="103"/>
+      <c r="E286" s="103" t="s">
         <v>840</v>
       </c>
-      <c r="F286" s="101"/>
-      <c r="G286" s="101"/>
-      <c r="H286" s="101"/>
+      <c r="F286" s="103"/>
+      <c r="G286" s="103"/>
+      <c r="H286" s="103"/>
     </row>
     <row r="287" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A287" s="100" t="s">
+      <c r="A287" s="104" t="s">
         <v>706</v>
       </c>
-      <c r="B287" s="100"/>
-      <c r="C287" s="100"/>
-      <c r="D287" s="100"/>
-      <c r="E287" s="100" t="s">
+      <c r="B287" s="104"/>
+      <c r="C287" s="104"/>
+      <c r="D287" s="104"/>
+      <c r="E287" s="104" t="s">
         <v>841</v>
       </c>
-      <c r="F287" s="100"/>
-      <c r="G287" s="100"/>
-      <c r="H287" s="100"/>
+      <c r="F287" s="104"/>
+      <c r="G287" s="104"/>
+      <c r="H287" s="104"/>
     </row>
     <row r="288" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A288" s="101" t="s">
+      <c r="A288" s="103" t="s">
         <v>595</v>
       </c>
-      <c r="B288" s="101"/>
-      <c r="C288" s="101"/>
-      <c r="D288" s="101"/>
-      <c r="E288" s="101" t="s">
+      <c r="B288" s="103"/>
+      <c r="C288" s="103"/>
+      <c r="D288" s="103"/>
+      <c r="E288" s="103" t="s">
         <v>842</v>
       </c>
-      <c r="F288" s="101"/>
-      <c r="G288" s="101"/>
-      <c r="H288" s="101"/>
+      <c r="F288" s="103"/>
+      <c r="G288" s="103"/>
+      <c r="H288" s="103"/>
     </row>
     <row r="289" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A289" s="100" t="s">
+      <c r="A289" s="104" t="s">
         <v>600</v>
       </c>
-      <c r="B289" s="100"/>
-      <c r="C289" s="100"/>
-      <c r="D289" s="100"/>
-      <c r="E289" s="100" t="s">
+      <c r="B289" s="104"/>
+      <c r="C289" s="104"/>
+      <c r="D289" s="104"/>
+      <c r="E289" s="104" t="s">
         <v>843</v>
       </c>
-      <c r="F289" s="100"/>
-      <c r="G289" s="100"/>
-      <c r="H289" s="100"/>
+      <c r="F289" s="104"/>
+      <c r="G289" s="104"/>
+      <c r="H289" s="104"/>
     </row>
     <row r="290" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A290" s="101" t="s">
+      <c r="A290" s="103" t="s">
         <v>605</v>
       </c>
-      <c r="B290" s="101"/>
-      <c r="C290" s="101"/>
-      <c r="D290" s="101"/>
-      <c r="E290" s="101" t="s">
+      <c r="B290" s="103"/>
+      <c r="C290" s="103"/>
+      <c r="D290" s="103"/>
+      <c r="E290" s="103" t="s">
         <v>844</v>
       </c>
-      <c r="F290" s="101"/>
-      <c r="G290" s="101"/>
-      <c r="H290" s="101"/>
+      <c r="F290" s="103"/>
+      <c r="G290" s="103"/>
+      <c r="H290" s="103"/>
     </row>
     <row r="291" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A291" s="100" t="s">
+      <c r="A291" s="104" t="s">
         <v>845</v>
       </c>
-      <c r="B291" s="100"/>
-      <c r="C291" s="100"/>
-      <c r="D291" s="100"/>
-      <c r="E291" s="100" t="s">
+      <c r="B291" s="104"/>
+      <c r="C291" s="104"/>
+      <c r="D291" s="104"/>
+      <c r="E291" s="104" t="s">
         <v>846</v>
       </c>
-      <c r="F291" s="100"/>
-      <c r="G291" s="100"/>
-      <c r="H291" s="100"/>
+      <c r="F291" s="104"/>
+      <c r="G291" s="104"/>
+      <c r="H291" s="104"/>
     </row>
     <row r="292" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A292" s="101" t="s">
+      <c r="A292" s="103" t="s">
         <v>847</v>
       </c>
-      <c r="B292" s="101"/>
-      <c r="C292" s="101"/>
-      <c r="D292" s="101"/>
-      <c r="E292" s="101" t="s">
+      <c r="B292" s="103"/>
+      <c r="C292" s="103"/>
+      <c r="D292" s="103"/>
+      <c r="E292" s="103" t="s">
         <v>848</v>
       </c>
-      <c r="F292" s="101"/>
-      <c r="G292" s="101"/>
-      <c r="H292" s="101"/>
+      <c r="F292" s="103"/>
+      <c r="G292" s="103"/>
+      <c r="H292" s="103"/>
     </row>
     <row r="293" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A293" s="100" t="s">
+      <c r="A293" s="104" t="s">
         <v>278</v>
       </c>
-      <c r="B293" s="100"/>
-      <c r="C293" s="100"/>
-      <c r="D293" s="100"/>
-      <c r="E293" s="100" t="s">
+      <c r="B293" s="104"/>
+      <c r="C293" s="104"/>
+      <c r="D293" s="104"/>
+      <c r="E293" s="104" t="s">
         <v>849</v>
       </c>
-      <c r="F293" s="100"/>
-      <c r="G293" s="100"/>
-      <c r="H293" s="100"/>
+      <c r="F293" s="104"/>
+      <c r="G293" s="104"/>
+      <c r="H293" s="104"/>
     </row>
     <row r="294" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A294" s="101" t="s">
+      <c r="A294" s="103" t="s">
         <v>272</v>
       </c>
-      <c r="B294" s="101"/>
-      <c r="C294" s="101"/>
-      <c r="D294" s="101"/>
-      <c r="E294" s="101" t="s">
+      <c r="B294" s="103"/>
+      <c r="C294" s="103"/>
+      <c r="D294" s="103"/>
+      <c r="E294" s="103" t="s">
         <v>850</v>
       </c>
-      <c r="F294" s="101"/>
-      <c r="G294" s="101"/>
-      <c r="H294" s="101"/>
+      <c r="F294" s="103"/>
+      <c r="G294" s="103"/>
+      <c r="H294" s="103"/>
     </row>
     <row r="295" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A295" s="100" t="s">
+      <c r="A295" s="104" t="s">
         <v>530</v>
       </c>
-      <c r="B295" s="100"/>
-      <c r="C295" s="100"/>
-      <c r="D295" s="100"/>
-      <c r="E295" s="100" t="s">
+      <c r="B295" s="104"/>
+      <c r="C295" s="104"/>
+      <c r="D295" s="104"/>
+      <c r="E295" s="104" t="s">
         <v>851</v>
       </c>
-      <c r="F295" s="100"/>
-      <c r="G295" s="100"/>
-      <c r="H295" s="100"/>
+      <c r="F295" s="104"/>
+      <c r="G295" s="104"/>
+      <c r="H295" s="104"/>
     </row>
     <row r="296" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A296" s="101" t="s">
+      <c r="A296" s="103" t="s">
         <v>610</v>
       </c>
-      <c r="B296" s="101"/>
-      <c r="C296" s="101"/>
-      <c r="D296" s="101"/>
-      <c r="E296" s="101" t="s">
+      <c r="B296" s="103"/>
+      <c r="C296" s="103"/>
+      <c r="D296" s="103"/>
+      <c r="E296" s="103" t="s">
         <v>852</v>
       </c>
-      <c r="F296" s="101"/>
-      <c r="G296" s="101"/>
-      <c r="H296" s="101"/>
+      <c r="F296" s="103"/>
+      <c r="G296" s="103"/>
+      <c r="H296" s="103"/>
     </row>
     <row r="297" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A297" s="100" t="s">
+      <c r="A297" s="104" t="s">
         <v>614</v>
       </c>
-      <c r="B297" s="100"/>
-      <c r="C297" s="100"/>
-      <c r="D297" s="100"/>
-      <c r="E297" s="100" t="s">
+      <c r="B297" s="104"/>
+      <c r="C297" s="104"/>
+      <c r="D297" s="104"/>
+      <c r="E297" s="104" t="s">
         <v>853</v>
       </c>
-      <c r="F297" s="100"/>
-      <c r="G297" s="100"/>
-      <c r="H297" s="100"/>
+      <c r="F297" s="104"/>
+      <c r="G297" s="104"/>
+      <c r="H297" s="104"/>
     </row>
     <row r="298" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A298" s="101" t="s">
+      <c r="A298" s="103" t="s">
         <v>618</v>
       </c>
-      <c r="B298" s="101"/>
-      <c r="C298" s="101"/>
-      <c r="D298" s="101"/>
-      <c r="E298" s="101" t="s">
+      <c r="B298" s="103"/>
+      <c r="C298" s="103"/>
+      <c r="D298" s="103"/>
+      <c r="E298" s="103" t="s">
         <v>854</v>
       </c>
-      <c r="F298" s="101"/>
-      <c r="G298" s="101"/>
-      <c r="H298" s="101"/>
+      <c r="F298" s="103"/>
+      <c r="G298" s="103"/>
+      <c r="H298" s="103"/>
     </row>
     <row r="299" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A299" s="100" t="s">
+      <c r="A299" s="104" t="s">
         <v>622</v>
       </c>
-      <c r="B299" s="100"/>
-      <c r="C299" s="100"/>
-      <c r="D299" s="100"/>
-      <c r="E299" s="100" t="s">
+      <c r="B299" s="104"/>
+      <c r="C299" s="104"/>
+      <c r="D299" s="104"/>
+      <c r="E299" s="104" t="s">
         <v>855</v>
       </c>
-      <c r="F299" s="100"/>
-      <c r="G299" s="100"/>
-      <c r="H299" s="100"/>
+      <c r="F299" s="104"/>
+      <c r="G299" s="104"/>
+      <c r="H299" s="104"/>
     </row>
     <row r="300" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A300" s="101" t="s">
+      <c r="A300" s="103" t="s">
         <v>626</v>
       </c>
-      <c r="B300" s="101"/>
-      <c r="C300" s="101"/>
-      <c r="D300" s="101"/>
-      <c r="E300" s="101" t="s">
+      <c r="B300" s="103"/>
+      <c r="C300" s="103"/>
+      <c r="D300" s="103"/>
+      <c r="E300" s="103" t="s">
         <v>856</v>
       </c>
-      <c r="F300" s="101"/>
-      <c r="G300" s="101"/>
-      <c r="H300" s="101"/>
+      <c r="F300" s="103"/>
+      <c r="G300" s="103"/>
+      <c r="H300" s="103"/>
     </row>
     <row r="301" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A301" s="100" t="s">
+      <c r="A301" s="104" t="s">
         <v>630</v>
       </c>
-      <c r="B301" s="100"/>
-      <c r="C301" s="100"/>
-      <c r="D301" s="100"/>
-      <c r="E301" s="100" t="s">
+      <c r="B301" s="104"/>
+      <c r="C301" s="104"/>
+      <c r="D301" s="104"/>
+      <c r="E301" s="104" t="s">
         <v>857</v>
       </c>
-      <c r="F301" s="100"/>
-      <c r="G301" s="100"/>
-      <c r="H301" s="100"/>
+      <c r="F301" s="104"/>
+      <c r="G301" s="104"/>
+      <c r="H301" s="104"/>
     </row>
     <row r="302" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A302" s="101" t="s">
+      <c r="A302" s="103" t="s">
         <v>858</v>
       </c>
-      <c r="B302" s="101"/>
-      <c r="C302" s="101"/>
-      <c r="D302" s="101"/>
-      <c r="E302" s="101" t="s">
+      <c r="B302" s="103"/>
+      <c r="C302" s="103"/>
+      <c r="D302" s="103"/>
+      <c r="E302" s="103" t="s">
         <v>859</v>
       </c>
-      <c r="F302" s="101"/>
-      <c r="G302" s="101"/>
-      <c r="H302" s="101"/>
+      <c r="F302" s="103"/>
+      <c r="G302" s="103"/>
+      <c r="H302" s="103"/>
     </row>
     <row r="303" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A303" s="100" t="s">
+      <c r="A303" s="104" t="s">
         <v>860</v>
       </c>
-      <c r="B303" s="100"/>
-      <c r="C303" s="100"/>
-      <c r="D303" s="100"/>
-      <c r="E303" s="100" t="s">
+      <c r="B303" s="104"/>
+      <c r="C303" s="104"/>
+      <c r="D303" s="104"/>
+      <c r="E303" s="104" t="s">
         <v>861</v>
       </c>
-      <c r="F303" s="100"/>
-      <c r="G303" s="100"/>
-      <c r="H303" s="100"/>
+      <c r="F303" s="104"/>
+      <c r="G303" s="104"/>
+      <c r="H303" s="104"/>
     </row>
     <row r="304" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A304" s="101" t="s">
+      <c r="A304" s="103" t="s">
         <v>862</v>
       </c>
-      <c r="B304" s="101"/>
-      <c r="C304" s="101"/>
-      <c r="D304" s="101"/>
-      <c r="E304" s="101" t="s">
+      <c r="B304" s="103"/>
+      <c r="C304" s="103"/>
+      <c r="D304" s="103"/>
+      <c r="E304" s="103" t="s">
         <v>863</v>
       </c>
-      <c r="F304" s="101"/>
-      <c r="G304" s="101"/>
-      <c r="H304" s="101"/>
+      <c r="F304" s="103"/>
+      <c r="G304" s="103"/>
+      <c r="H304" s="103"/>
     </row>
     <row r="305" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A305" s="100" t="s">
+      <c r="A305" s="104" t="s">
         <v>864</v>
       </c>
-      <c r="B305" s="100"/>
-      <c r="C305" s="100"/>
-      <c r="D305" s="100"/>
-      <c r="E305" s="100" t="s">
+      <c r="B305" s="104"/>
+      <c r="C305" s="104"/>
+      <c r="D305" s="104"/>
+      <c r="E305" s="104" t="s">
         <v>865</v>
       </c>
-      <c r="F305" s="100"/>
-      <c r="G305" s="100"/>
-      <c r="H305" s="100"/>
+      <c r="F305" s="104"/>
+      <c r="G305" s="104"/>
+      <c r="H305" s="104"/>
     </row>
     <row r="306" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A306" s="101" t="s">
+      <c r="A306" s="103" t="s">
         <v>866</v>
       </c>
-      <c r="B306" s="101"/>
-      <c r="C306" s="101"/>
-      <c r="D306" s="101"/>
-      <c r="E306" s="101" t="s">
+      <c r="B306" s="103"/>
+      <c r="C306" s="103"/>
+      <c r="D306" s="103"/>
+      <c r="E306" s="103" t="s">
         <v>867</v>
       </c>
-      <c r="F306" s="101"/>
-      <c r="G306" s="101"/>
-      <c r="H306" s="101"/>
+      <c r="F306" s="103"/>
+      <c r="G306" s="103"/>
+      <c r="H306" s="103"/>
     </row>
     <row r="307" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A307" s="100" t="s">
+      <c r="A307" s="104" t="s">
         <v>868</v>
       </c>
-      <c r="B307" s="100"/>
-      <c r="C307" s="100"/>
-      <c r="D307" s="100"/>
-      <c r="E307" s="100" t="s">
+      <c r="B307" s="104"/>
+      <c r="C307" s="104"/>
+      <c r="D307" s="104"/>
+      <c r="E307" s="104" t="s">
         <v>869</v>
       </c>
-      <c r="F307" s="100"/>
-      <c r="G307" s="100"/>
-      <c r="H307" s="100"/>
+      <c r="F307" s="104"/>
+      <c r="G307" s="104"/>
+      <c r="H307" s="104"/>
     </row>
     <row r="308" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A308" s="101" t="s">
+      <c r="A308" s="103" t="s">
         <v>870</v>
       </c>
-      <c r="B308" s="101"/>
-      <c r="C308" s="101"/>
-      <c r="D308" s="101"/>
-      <c r="E308" s="101" t="s">
+      <c r="B308" s="103"/>
+      <c r="C308" s="103"/>
+      <c r="D308" s="103"/>
+      <c r="E308" s="103" t="s">
         <v>871</v>
       </c>
-      <c r="F308" s="101"/>
-      <c r="G308" s="101"/>
-      <c r="H308" s="101"/>
+      <c r="F308" s="103"/>
+      <c r="G308" s="103"/>
+      <c r="H308" s="103"/>
     </row>
     <row r="309" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A309" s="100" t="s">
+      <c r="A309" s="104" t="s">
         <v>872</v>
       </c>
-      <c r="B309" s="100"/>
-      <c r="C309" s="100"/>
-      <c r="D309" s="100"/>
-      <c r="E309" s="100" t="s">
+      <c r="B309" s="104"/>
+      <c r="C309" s="104"/>
+      <c r="D309" s="104"/>
+      <c r="E309" s="104" t="s">
         <v>873</v>
       </c>
-      <c r="F309" s="100"/>
-      <c r="G309" s="100"/>
-      <c r="H309" s="100"/>
+      <c r="F309" s="104"/>
+      <c r="G309" s="104"/>
+      <c r="H309" s="104"/>
     </row>
     <row r="310" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A310" s="101" t="s">
+      <c r="A310" s="103" t="s">
         <v>874</v>
       </c>
-      <c r="B310" s="101"/>
-      <c r="C310" s="101"/>
-      <c r="D310" s="101"/>
-      <c r="E310" s="101" t="s">
+      <c r="B310" s="103"/>
+      <c r="C310" s="103"/>
+      <c r="D310" s="103"/>
+      <c r="E310" s="103" t="s">
         <v>875</v>
       </c>
-      <c r="F310" s="101"/>
-      <c r="G310" s="101"/>
-      <c r="H310" s="101"/>
+      <c r="F310" s="103"/>
+      <c r="G310" s="103"/>
+      <c r="H310" s="103"/>
     </row>
     <row r="311" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A311" s="100" t="s">
+      <c r="A311" s="104" t="s">
         <v>876</v>
       </c>
-      <c r="B311" s="100"/>
-      <c r="C311" s="100"/>
-      <c r="D311" s="100"/>
-      <c r="E311" s="100" t="s">
+      <c r="B311" s="104"/>
+      <c r="C311" s="104"/>
+      <c r="D311" s="104"/>
+      <c r="E311" s="104" t="s">
         <v>877</v>
       </c>
-      <c r="F311" s="100"/>
-      <c r="G311" s="100"/>
-      <c r="H311" s="100"/>
+      <c r="F311" s="104"/>
+      <c r="G311" s="104"/>
+      <c r="H311" s="104"/>
     </row>
     <row r="312" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A312" s="101" t="s">
+      <c r="A312" s="103" t="s">
         <v>878</v>
       </c>
-      <c r="B312" s="101"/>
-      <c r="C312" s="101"/>
-      <c r="D312" s="101"/>
-      <c r="E312" s="101" t="s">
+      <c r="B312" s="103"/>
+      <c r="C312" s="103"/>
+      <c r="D312" s="103"/>
+      <c r="E312" s="103" t="s">
         <v>879</v>
       </c>
-      <c r="F312" s="101"/>
-      <c r="G312" s="101"/>
-      <c r="H312" s="101"/>
+      <c r="F312" s="103"/>
+      <c r="G312" s="103"/>
+      <c r="H312" s="103"/>
     </row>
     <row r="313" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A313" s="100" t="s">
+      <c r="A313" s="104" t="s">
         <v>880</v>
       </c>
-      <c r="B313" s="100"/>
-      <c r="C313" s="100"/>
-      <c r="D313" s="100"/>
-      <c r="E313" s="100" t="s">
+      <c r="B313" s="104"/>
+      <c r="C313" s="104"/>
+      <c r="D313" s="104"/>
+      <c r="E313" s="104" t="s">
         <v>881</v>
       </c>
-      <c r="F313" s="100"/>
-      <c r="G313" s="100"/>
-      <c r="H313" s="100"/>
+      <c r="F313" s="104"/>
+      <c r="G313" s="104"/>
+      <c r="H313" s="104"/>
     </row>
     <row r="314" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A314" s="101" t="s">
+      <c r="A314" s="103" t="s">
         <v>882</v>
       </c>
-      <c r="B314" s="101"/>
-      <c r="C314" s="101"/>
-      <c r="D314" s="101"/>
-      <c r="E314" s="101" t="s">
+      <c r="B314" s="103"/>
+      <c r="C314" s="103"/>
+      <c r="D314" s="103"/>
+      <c r="E314" s="103" t="s">
         <v>883</v>
       </c>
-      <c r="F314" s="101"/>
-      <c r="G314" s="101"/>
-      <c r="H314" s="101"/>
+      <c r="F314" s="103"/>
+      <c r="G314" s="103"/>
+      <c r="H314" s="103"/>
     </row>
     <row r="315" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A315" s="100" t="s">
+      <c r="A315" s="104" t="s">
         <v>884</v>
       </c>
-      <c r="B315" s="100"/>
-      <c r="C315" s="100"/>
-      <c r="D315" s="100"/>
-      <c r="E315" s="100" t="s">
+      <c r="B315" s="104"/>
+      <c r="C315" s="104"/>
+      <c r="D315" s="104"/>
+      <c r="E315" s="104" t="s">
         <v>885</v>
       </c>
-      <c r="F315" s="100"/>
-      <c r="G315" s="100"/>
-      <c r="H315" s="100"/>
+      <c r="F315" s="104"/>
+      <c r="G315" s="104"/>
+      <c r="H315" s="104"/>
     </row>
     <row r="316" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A316" s="101" t="s">
+      <c r="A316" s="103" t="s">
         <v>886</v>
       </c>
-      <c r="B316" s="101"/>
-      <c r="C316" s="101"/>
-      <c r="D316" s="101"/>
-      <c r="E316" s="101" t="s">
+      <c r="B316" s="103"/>
+      <c r="C316" s="103"/>
+      <c r="D316" s="103"/>
+      <c r="E316" s="103" t="s">
         <v>887</v>
       </c>
-      <c r="F316" s="101"/>
-      <c r="G316" s="101"/>
-      <c r="H316" s="101"/>
+      <c r="F316" s="103"/>
+      <c r="G316" s="103"/>
+      <c r="H316" s="103"/>
     </row>
     <row r="317" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A317" s="100" t="s">
+      <c r="A317" s="104" t="s">
         <v>888</v>
       </c>
-      <c r="B317" s="100"/>
-      <c r="C317" s="100"/>
-      <c r="D317" s="100"/>
-      <c r="E317" s="100" t="s">
+      <c r="B317" s="104"/>
+      <c r="C317" s="104"/>
+      <c r="D317" s="104"/>
+      <c r="E317" s="104" t="s">
         <v>889</v>
       </c>
-      <c r="F317" s="100"/>
-      <c r="G317" s="100"/>
-      <c r="H317" s="100"/>
+      <c r="F317" s="104"/>
+      <c r="G317" s="104"/>
+      <c r="H317" s="104"/>
     </row>
     <row r="318" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A318" s="101" t="s">
+      <c r="A318" s="103" t="s">
         <v>890</v>
       </c>
-      <c r="B318" s="101"/>
-      <c r="C318" s="101"/>
-      <c r="D318" s="101"/>
-      <c r="E318" s="101" t="s">
+      <c r="B318" s="103"/>
+      <c r="C318" s="103"/>
+      <c r="D318" s="103"/>
+      <c r="E318" s="103" t="s">
         <v>891</v>
       </c>
-      <c r="F318" s="101"/>
-      <c r="G318" s="101"/>
-      <c r="H318" s="101"/>
+      <c r="F318" s="103"/>
+      <c r="G318" s="103"/>
+      <c r="H318" s="103"/>
     </row>
     <row r="319" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A319" s="100" t="s">
+      <c r="A319" s="104" t="s">
         <v>892</v>
       </c>
-      <c r="B319" s="100"/>
-      <c r="C319" s="100"/>
-      <c r="D319" s="100"/>
-      <c r="E319" s="100" t="s">
+      <c r="B319" s="104"/>
+      <c r="C319" s="104"/>
+      <c r="D319" s="104"/>
+      <c r="E319" s="104" t="s">
         <v>893</v>
       </c>
-      <c r="F319" s="100"/>
-      <c r="G319" s="100"/>
-      <c r="H319" s="100"/>
+      <c r="F319" s="104"/>
+      <c r="G319" s="104"/>
+      <c r="H319" s="104"/>
     </row>
     <row r="320" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A320" s="101" t="s">
+      <c r="A320" s="103" t="s">
         <v>894</v>
       </c>
-      <c r="B320" s="101"/>
-      <c r="C320" s="101"/>
-      <c r="D320" s="101"/>
-      <c r="E320" s="101" t="s">
+      <c r="B320" s="103"/>
+      <c r="C320" s="103"/>
+      <c r="D320" s="103"/>
+      <c r="E320" s="103" t="s">
         <v>895</v>
       </c>
-      <c r="F320" s="101"/>
-      <c r="G320" s="101"/>
-      <c r="H320" s="101"/>
+      <c r="F320" s="103"/>
+      <c r="G320" s="103"/>
+      <c r="H320" s="103"/>
     </row>
     <row r="321" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A321" s="100" t="s">
+      <c r="A321" s="104" t="s">
         <v>896</v>
       </c>
-      <c r="B321" s="100"/>
-      <c r="C321" s="100"/>
-      <c r="D321" s="100"/>
-      <c r="E321" s="100" t="s">
+      <c r="B321" s="104"/>
+      <c r="C321" s="104"/>
+      <c r="D321" s="104"/>
+      <c r="E321" s="104" t="s">
         <v>897</v>
       </c>
-      <c r="F321" s="100"/>
-      <c r="G321" s="100"/>
-      <c r="H321" s="100"/>
+      <c r="F321" s="104"/>
+      <c r="G321" s="104"/>
+      <c r="H321" s="104"/>
     </row>
     <row r="322" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A322" s="116" t="s">
+      <c r="A322" s="105" t="s">
         <v>898</v>
       </c>
-      <c r="B322" s="116"/>
-      <c r="C322" s="116"/>
-      <c r="D322" s="116"/>
-      <c r="E322" s="116" t="s">
+      <c r="B322" s="105"/>
+      <c r="C322" s="105"/>
+      <c r="D322" s="105"/>
+      <c r="E322" s="105" t="s">
         <v>899</v>
       </c>
-      <c r="F322" s="116"/>
-      <c r="G322" s="116"/>
-      <c r="H322" s="116"/>
+      <c r="F322" s="105"/>
+      <c r="G322" s="105"/>
+      <c r="H322" s="105"/>
     </row>
     <row r="325" spans="1:8" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A325" s="104" t="s">
+      <c r="A325" s="91" t="s">
         <v>900</v>
       </c>
-      <c r="B325" s="104"/>
-      <c r="C325" s="104"/>
-      <c r="D325" s="104"/>
-      <c r="E325" s="104"/>
-      <c r="F325" s="104"/>
-      <c r="G325" s="104"/>
-      <c r="H325" s="104"/>
+      <c r="B325" s="91"/>
+      <c r="C325" s="91"/>
+      <c r="D325" s="91"/>
+      <c r="E325" s="91"/>
+      <c r="F325" s="91"/>
+      <c r="G325" s="91"/>
+      <c r="H325" s="91"/>
     </row>
     <row r="326" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A326" s="105" t="s">
+      <c r="A326" s="92" t="s">
         <v>901</v>
       </c>
-      <c r="B326" s="105"/>
-      <c r="C326" s="105"/>
-      <c r="D326" s="105"/>
-      <c r="E326" s="105"/>
-      <c r="F326" s="105"/>
-      <c r="G326" s="105"/>
-      <c r="H326" s="105"/>
+      <c r="B326" s="92"/>
+      <c r="C326" s="92"/>
+      <c r="D326" s="92"/>
+      <c r="E326" s="92"/>
+      <c r="F326" s="92"/>
+      <c r="G326" s="92"/>
+      <c r="H326" s="92"/>
     </row>
     <row r="327" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A327" s="105"/>
-      <c r="B327" s="105"/>
-      <c r="C327" s="105"/>
-      <c r="D327" s="105"/>
-      <c r="E327" s="105"/>
-      <c r="F327" s="105"/>
-      <c r="G327" s="105"/>
-      <c r="H327" s="105"/>
+      <c r="A327" s="92"/>
+      <c r="B327" s="92"/>
+      <c r="C327" s="92"/>
+      <c r="D327" s="92"/>
+      <c r="E327" s="92"/>
+      <c r="F327" s="92"/>
+      <c r="G327" s="92"/>
+      <c r="H327" s="92"/>
     </row>
     <row r="328" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A328" s="40"/>
@@ -16258,16 +16258,16 @@
       <c r="H328" s="40"/>
     </row>
     <row r="329" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A329" s="106" t="s">
+      <c r="A329" s="93" t="s">
         <v>902</v>
       </c>
-      <c r="B329" s="106"/>
-      <c r="C329" s="106"/>
-      <c r="D329" s="106"/>
-      <c r="E329" s="106"/>
-      <c r="F329" s="106"/>
-      <c r="G329" s="106"/>
-      <c r="H329" s="106"/>
+      <c r="B329" s="93"/>
+      <c r="C329" s="93"/>
+      <c r="D329" s="93"/>
+      <c r="E329" s="93"/>
+      <c r="F329" s="93"/>
+      <c r="G329" s="93"/>
+      <c r="H329" s="93"/>
     </row>
     <row r="330" spans="1:8" ht="24" x14ac:dyDescent="0.25">
       <c r="A330" s="41" t="s">
@@ -16566,16 +16566,16 @@
       <c r="H341" s="40"/>
     </row>
     <row r="342" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A342" s="106" t="s">
+      <c r="A342" s="93" t="s">
         <v>975</v>
       </c>
-      <c r="B342" s="106"/>
-      <c r="C342" s="106"/>
-      <c r="D342" s="106"/>
-      <c r="E342" s="106"/>
-      <c r="F342" s="106"/>
-      <c r="G342" s="106"/>
-      <c r="H342" s="106"/>
+      <c r="B342" s="93"/>
+      <c r="C342" s="93"/>
+      <c r="D342" s="93"/>
+      <c r="E342" s="93"/>
+      <c r="F342" s="93"/>
+      <c r="G342" s="93"/>
+      <c r="H342" s="93"/>
     </row>
     <row r="343" spans="1:8" ht="24" x14ac:dyDescent="0.25">
       <c r="A343" s="41" t="s">
@@ -16822,73 +16822,230 @@
       <c r="H352" s="40"/>
     </row>
     <row r="353" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A353" s="106" t="s">
+      <c r="A353" s="93" t="s">
         <v>1036</v>
       </c>
-      <c r="B353" s="106"/>
-      <c r="C353" s="106"/>
-      <c r="D353" s="106"/>
-      <c r="E353" s="106"/>
-      <c r="F353" s="106"/>
-      <c r="G353" s="106"/>
-      <c r="H353" s="106"/>
+      <c r="B353" s="93"/>
+      <c r="C353" s="93"/>
+      <c r="D353" s="93"/>
+      <c r="E353" s="93"/>
+      <c r="F353" s="93"/>
+      <c r="G353" s="93"/>
+      <c r="H353" s="93"/>
     </row>
     <row r="354" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A354" s="107" t="s">
+      <c r="A354" s="94" t="s">
         <v>1037</v>
       </c>
-      <c r="B354" s="108"/>
-      <c r="C354" s="108"/>
-      <c r="D354" s="108"/>
-      <c r="E354" s="108"/>
-      <c r="F354" s="108"/>
-      <c r="G354" s="108"/>
-      <c r="H354" s="109"/>
+      <c r="B354" s="95"/>
+      <c r="C354" s="95"/>
+      <c r="D354" s="95"/>
+      <c r="E354" s="95"/>
+      <c r="F354" s="95"/>
+      <c r="G354" s="95"/>
+      <c r="H354" s="96"/>
     </row>
     <row r="355" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A355" s="110"/>
-      <c r="B355" s="111"/>
-      <c r="C355" s="111"/>
-      <c r="D355" s="111"/>
-      <c r="E355" s="111"/>
-      <c r="F355" s="111"/>
-      <c r="G355" s="111"/>
-      <c r="H355" s="112"/>
+      <c r="A355" s="97"/>
+      <c r="B355" s="98"/>
+      <c r="C355" s="98"/>
+      <c r="D355" s="98"/>
+      <c r="E355" s="98"/>
+      <c r="F355" s="98"/>
+      <c r="G355" s="98"/>
+      <c r="H355" s="99"/>
     </row>
     <row r="356" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A356" s="113"/>
-      <c r="B356" s="114"/>
-      <c r="C356" s="114"/>
-      <c r="D356" s="114"/>
-      <c r="E356" s="114"/>
-      <c r="F356" s="114"/>
-      <c r="G356" s="114"/>
-      <c r="H356" s="115"/>
+      <c r="A356" s="100"/>
+      <c r="B356" s="101"/>
+      <c r="C356" s="101"/>
+      <c r="D356" s="101"/>
+      <c r="E356" s="101"/>
+      <c r="F356" s="101"/>
+      <c r="G356" s="101"/>
+      <c r="H356" s="102"/>
     </row>
     <row r="357" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A357" s="103" t="s">
+      <c r="A357" s="90" t="s">
         <v>1038</v>
       </c>
-      <c r="B357" s="103"/>
-      <c r="C357" s="103"/>
-      <c r="D357" s="103"/>
-      <c r="E357" s="103"/>
-      <c r="F357" s="103"/>
-      <c r="G357" s="103"/>
-      <c r="H357" s="103"/>
+      <c r="B357" s="90"/>
+      <c r="C357" s="90"/>
+      <c r="D357" s="90"/>
+      <c r="E357" s="90"/>
+      <c r="F357" s="90"/>
+      <c r="G357" s="90"/>
+      <c r="H357" s="90"/>
     </row>
     <row r="358" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A358" s="103"/>
-      <c r="B358" s="103"/>
-      <c r="C358" s="103"/>
-      <c r="D358" s="103"/>
-      <c r="E358" s="103"/>
-      <c r="F358" s="103"/>
-      <c r="G358" s="103"/>
-      <c r="H358" s="103"/>
+      <c r="A358" s="90"/>
+      <c r="B358" s="90"/>
+      <c r="C358" s="90"/>
+      <c r="D358" s="90"/>
+      <c r="E358" s="90"/>
+      <c r="F358" s="90"/>
+      <c r="G358" s="90"/>
+      <c r="H358" s="90"/>
     </row>
   </sheetData>
   <mergeCells count="170">
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="A50:H50"/>
+    <mergeCell ref="A63:H63"/>
+    <mergeCell ref="A75:H75"/>
+    <mergeCell ref="A88:H88"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A5:H7"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="C156:H156"/>
+    <mergeCell ref="C157:H157"/>
+    <mergeCell ref="C158:H158"/>
+    <mergeCell ref="C159:H159"/>
+    <mergeCell ref="A161:H161"/>
+    <mergeCell ref="A172:H172"/>
+    <mergeCell ref="A105:H105"/>
+    <mergeCell ref="A107:H107"/>
+    <mergeCell ref="A108:H109"/>
+    <mergeCell ref="A153:H153"/>
+    <mergeCell ref="C154:H154"/>
+    <mergeCell ref="C155:H155"/>
+    <mergeCell ref="D191:H191"/>
+    <mergeCell ref="A193:H193"/>
+    <mergeCell ref="A194:H194"/>
+    <mergeCell ref="A254:H254"/>
+    <mergeCell ref="A255:H255"/>
+    <mergeCell ref="A257:H257"/>
+    <mergeCell ref="A173:H175"/>
+    <mergeCell ref="A186:H186"/>
+    <mergeCell ref="D187:H187"/>
+    <mergeCell ref="D188:H188"/>
+    <mergeCell ref="D189:H189"/>
+    <mergeCell ref="D190:H190"/>
+    <mergeCell ref="A263:D263"/>
+    <mergeCell ref="E263:H263"/>
+    <mergeCell ref="A264:D264"/>
+    <mergeCell ref="E264:H264"/>
+    <mergeCell ref="A265:D265"/>
+    <mergeCell ref="E265:H265"/>
+    <mergeCell ref="A258:H258"/>
+    <mergeCell ref="A260:D260"/>
+    <mergeCell ref="E260:H260"/>
+    <mergeCell ref="A261:D261"/>
+    <mergeCell ref="E261:H261"/>
+    <mergeCell ref="A262:D262"/>
+    <mergeCell ref="E262:H262"/>
+    <mergeCell ref="A269:D269"/>
+    <mergeCell ref="E269:H269"/>
+    <mergeCell ref="A270:D270"/>
+    <mergeCell ref="E270:H270"/>
+    <mergeCell ref="A271:D271"/>
+    <mergeCell ref="E271:H271"/>
+    <mergeCell ref="A266:D266"/>
+    <mergeCell ref="E266:H266"/>
+    <mergeCell ref="A267:D267"/>
+    <mergeCell ref="E267:H267"/>
+    <mergeCell ref="A268:D268"/>
+    <mergeCell ref="E268:H268"/>
+    <mergeCell ref="A275:D275"/>
+    <mergeCell ref="E275:H275"/>
+    <mergeCell ref="A276:D276"/>
+    <mergeCell ref="E276:H276"/>
+    <mergeCell ref="A277:D277"/>
+    <mergeCell ref="E277:H277"/>
+    <mergeCell ref="A272:D272"/>
+    <mergeCell ref="E272:H272"/>
+    <mergeCell ref="A273:D273"/>
+    <mergeCell ref="E273:H273"/>
+    <mergeCell ref="A274:D274"/>
+    <mergeCell ref="E274:H274"/>
+    <mergeCell ref="A281:D281"/>
+    <mergeCell ref="E281:H281"/>
+    <mergeCell ref="A282:D282"/>
+    <mergeCell ref="E282:H282"/>
+    <mergeCell ref="A283:D283"/>
+    <mergeCell ref="E283:H283"/>
+    <mergeCell ref="A278:D278"/>
+    <mergeCell ref="E278:H278"/>
+    <mergeCell ref="A279:D279"/>
+    <mergeCell ref="E279:H279"/>
+    <mergeCell ref="A280:D280"/>
+    <mergeCell ref="E280:H280"/>
+    <mergeCell ref="A287:D287"/>
+    <mergeCell ref="E287:H287"/>
+    <mergeCell ref="A288:D288"/>
+    <mergeCell ref="E288:H288"/>
+    <mergeCell ref="A289:D289"/>
+    <mergeCell ref="E289:H289"/>
+    <mergeCell ref="A284:D284"/>
+    <mergeCell ref="E284:H284"/>
+    <mergeCell ref="A285:D285"/>
+    <mergeCell ref="E285:H285"/>
+    <mergeCell ref="A286:D286"/>
+    <mergeCell ref="E286:H286"/>
+    <mergeCell ref="A293:D293"/>
+    <mergeCell ref="E293:H293"/>
+    <mergeCell ref="A294:D294"/>
+    <mergeCell ref="E294:H294"/>
+    <mergeCell ref="A295:D295"/>
+    <mergeCell ref="E295:H295"/>
+    <mergeCell ref="A290:D290"/>
+    <mergeCell ref="E290:H290"/>
+    <mergeCell ref="A291:D291"/>
+    <mergeCell ref="E291:H291"/>
+    <mergeCell ref="A292:D292"/>
+    <mergeCell ref="E292:H292"/>
+    <mergeCell ref="A299:D299"/>
+    <mergeCell ref="E299:H299"/>
+    <mergeCell ref="A300:D300"/>
+    <mergeCell ref="E300:H300"/>
+    <mergeCell ref="A301:D301"/>
+    <mergeCell ref="E301:H301"/>
+    <mergeCell ref="A296:D296"/>
+    <mergeCell ref="E296:H296"/>
+    <mergeCell ref="A297:D297"/>
+    <mergeCell ref="E297:H297"/>
+    <mergeCell ref="A298:D298"/>
+    <mergeCell ref="E298:H298"/>
+    <mergeCell ref="A305:D305"/>
+    <mergeCell ref="E305:H305"/>
+    <mergeCell ref="A306:D306"/>
+    <mergeCell ref="E306:H306"/>
+    <mergeCell ref="A307:D307"/>
+    <mergeCell ref="E307:H307"/>
+    <mergeCell ref="A302:D302"/>
+    <mergeCell ref="E302:H302"/>
+    <mergeCell ref="A303:D303"/>
+    <mergeCell ref="E303:H303"/>
+    <mergeCell ref="A304:D304"/>
+    <mergeCell ref="E304:H304"/>
+    <mergeCell ref="A311:D311"/>
+    <mergeCell ref="E311:H311"/>
+    <mergeCell ref="A312:D312"/>
+    <mergeCell ref="E312:H312"/>
+    <mergeCell ref="A313:D313"/>
+    <mergeCell ref="E313:H313"/>
+    <mergeCell ref="A308:D308"/>
+    <mergeCell ref="E308:H308"/>
+    <mergeCell ref="A309:D309"/>
+    <mergeCell ref="E309:H309"/>
+    <mergeCell ref="A310:D310"/>
+    <mergeCell ref="E310:H310"/>
+    <mergeCell ref="A317:D317"/>
+    <mergeCell ref="E317:H317"/>
+    <mergeCell ref="A318:D318"/>
+    <mergeCell ref="E318:H318"/>
+    <mergeCell ref="A319:D319"/>
+    <mergeCell ref="E319:H319"/>
+    <mergeCell ref="A314:D314"/>
+    <mergeCell ref="E314:H314"/>
+    <mergeCell ref="A315:D315"/>
+    <mergeCell ref="E315:H315"/>
+    <mergeCell ref="A316:D316"/>
+    <mergeCell ref="E316:H316"/>
     <mergeCell ref="A357:H358"/>
     <mergeCell ref="A325:H325"/>
     <mergeCell ref="A326:H327"/>
@@ -16902,163 +17059,6 @@
     <mergeCell ref="E321:H321"/>
     <mergeCell ref="A322:D322"/>
     <mergeCell ref="E322:H322"/>
-    <mergeCell ref="A317:D317"/>
-    <mergeCell ref="E317:H317"/>
-    <mergeCell ref="A318:D318"/>
-    <mergeCell ref="E318:H318"/>
-    <mergeCell ref="A319:D319"/>
-    <mergeCell ref="E319:H319"/>
-    <mergeCell ref="A314:D314"/>
-    <mergeCell ref="E314:H314"/>
-    <mergeCell ref="A315:D315"/>
-    <mergeCell ref="E315:H315"/>
-    <mergeCell ref="A316:D316"/>
-    <mergeCell ref="E316:H316"/>
-    <mergeCell ref="A311:D311"/>
-    <mergeCell ref="E311:H311"/>
-    <mergeCell ref="A312:D312"/>
-    <mergeCell ref="E312:H312"/>
-    <mergeCell ref="A313:D313"/>
-    <mergeCell ref="E313:H313"/>
-    <mergeCell ref="A308:D308"/>
-    <mergeCell ref="E308:H308"/>
-    <mergeCell ref="A309:D309"/>
-    <mergeCell ref="E309:H309"/>
-    <mergeCell ref="A310:D310"/>
-    <mergeCell ref="E310:H310"/>
-    <mergeCell ref="A305:D305"/>
-    <mergeCell ref="E305:H305"/>
-    <mergeCell ref="A306:D306"/>
-    <mergeCell ref="E306:H306"/>
-    <mergeCell ref="A307:D307"/>
-    <mergeCell ref="E307:H307"/>
-    <mergeCell ref="A302:D302"/>
-    <mergeCell ref="E302:H302"/>
-    <mergeCell ref="A303:D303"/>
-    <mergeCell ref="E303:H303"/>
-    <mergeCell ref="A304:D304"/>
-    <mergeCell ref="E304:H304"/>
-    <mergeCell ref="A299:D299"/>
-    <mergeCell ref="E299:H299"/>
-    <mergeCell ref="A300:D300"/>
-    <mergeCell ref="E300:H300"/>
-    <mergeCell ref="A301:D301"/>
-    <mergeCell ref="E301:H301"/>
-    <mergeCell ref="A296:D296"/>
-    <mergeCell ref="E296:H296"/>
-    <mergeCell ref="A297:D297"/>
-    <mergeCell ref="E297:H297"/>
-    <mergeCell ref="A298:D298"/>
-    <mergeCell ref="E298:H298"/>
-    <mergeCell ref="A293:D293"/>
-    <mergeCell ref="E293:H293"/>
-    <mergeCell ref="A294:D294"/>
-    <mergeCell ref="E294:H294"/>
-    <mergeCell ref="A295:D295"/>
-    <mergeCell ref="E295:H295"/>
-    <mergeCell ref="A290:D290"/>
-    <mergeCell ref="E290:H290"/>
-    <mergeCell ref="A291:D291"/>
-    <mergeCell ref="E291:H291"/>
-    <mergeCell ref="A292:D292"/>
-    <mergeCell ref="E292:H292"/>
-    <mergeCell ref="A287:D287"/>
-    <mergeCell ref="E287:H287"/>
-    <mergeCell ref="A288:D288"/>
-    <mergeCell ref="E288:H288"/>
-    <mergeCell ref="A289:D289"/>
-    <mergeCell ref="E289:H289"/>
-    <mergeCell ref="A284:D284"/>
-    <mergeCell ref="E284:H284"/>
-    <mergeCell ref="A285:D285"/>
-    <mergeCell ref="E285:H285"/>
-    <mergeCell ref="A286:D286"/>
-    <mergeCell ref="E286:H286"/>
-    <mergeCell ref="A281:D281"/>
-    <mergeCell ref="E281:H281"/>
-    <mergeCell ref="A282:D282"/>
-    <mergeCell ref="E282:H282"/>
-    <mergeCell ref="A283:D283"/>
-    <mergeCell ref="E283:H283"/>
-    <mergeCell ref="A278:D278"/>
-    <mergeCell ref="E278:H278"/>
-    <mergeCell ref="A279:D279"/>
-    <mergeCell ref="E279:H279"/>
-    <mergeCell ref="A280:D280"/>
-    <mergeCell ref="E280:H280"/>
-    <mergeCell ref="A275:D275"/>
-    <mergeCell ref="E275:H275"/>
-    <mergeCell ref="A276:D276"/>
-    <mergeCell ref="E276:H276"/>
-    <mergeCell ref="A277:D277"/>
-    <mergeCell ref="E277:H277"/>
-    <mergeCell ref="A272:D272"/>
-    <mergeCell ref="E272:H272"/>
-    <mergeCell ref="A273:D273"/>
-    <mergeCell ref="E273:H273"/>
-    <mergeCell ref="A274:D274"/>
-    <mergeCell ref="E274:H274"/>
-    <mergeCell ref="A269:D269"/>
-    <mergeCell ref="E269:H269"/>
-    <mergeCell ref="A270:D270"/>
-    <mergeCell ref="E270:H270"/>
-    <mergeCell ref="A271:D271"/>
-    <mergeCell ref="E271:H271"/>
-    <mergeCell ref="A266:D266"/>
-    <mergeCell ref="E266:H266"/>
-    <mergeCell ref="A267:D267"/>
-    <mergeCell ref="E267:H267"/>
-    <mergeCell ref="A268:D268"/>
-    <mergeCell ref="E268:H268"/>
-    <mergeCell ref="A263:D263"/>
-    <mergeCell ref="E263:H263"/>
-    <mergeCell ref="A264:D264"/>
-    <mergeCell ref="E264:H264"/>
-    <mergeCell ref="A265:D265"/>
-    <mergeCell ref="E265:H265"/>
-    <mergeCell ref="A258:H258"/>
-    <mergeCell ref="A260:D260"/>
-    <mergeCell ref="E260:H260"/>
-    <mergeCell ref="A261:D261"/>
-    <mergeCell ref="E261:H261"/>
-    <mergeCell ref="A262:D262"/>
-    <mergeCell ref="E262:H262"/>
-    <mergeCell ref="D191:H191"/>
-    <mergeCell ref="A193:H193"/>
-    <mergeCell ref="A194:H194"/>
-    <mergeCell ref="A254:H254"/>
-    <mergeCell ref="A255:H255"/>
-    <mergeCell ref="A257:H257"/>
-    <mergeCell ref="A173:H175"/>
-    <mergeCell ref="A186:H186"/>
-    <mergeCell ref="D187:H187"/>
-    <mergeCell ref="D188:H188"/>
-    <mergeCell ref="D189:H189"/>
-    <mergeCell ref="D190:H190"/>
-    <mergeCell ref="C156:H156"/>
-    <mergeCell ref="C157:H157"/>
-    <mergeCell ref="C158:H158"/>
-    <mergeCell ref="C159:H159"/>
-    <mergeCell ref="A161:H161"/>
-    <mergeCell ref="A172:H172"/>
-    <mergeCell ref="A105:H105"/>
-    <mergeCell ref="A107:H107"/>
-    <mergeCell ref="A108:H109"/>
-    <mergeCell ref="A153:H153"/>
-    <mergeCell ref="C154:H154"/>
-    <mergeCell ref="C155:H155"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="A39:H39"/>
-    <mergeCell ref="A50:H50"/>
-    <mergeCell ref="A63:H63"/>
-    <mergeCell ref="A75:H75"/>
-    <mergeCell ref="A88:H88"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A5:H7"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A16:H16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -17086,13 +17086,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="88" t="s">
+      <c r="A1" s="78" t="s">
         <v>1039</v>
       </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
     </row>
     <row r="2" spans="1:9" ht="15" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:9" ht="15" x14ac:dyDescent="0.25">
@@ -17207,13 +17207,13 @@
     </row>
     <row r="9" spans="1:9" ht="15" x14ac:dyDescent="0.25"/>
     <row r="10" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A10" s="89" t="s">
+      <c r="A10" s="79" t="s">
         <v>1064</v>
       </c>
-      <c r="B10" s="89"/>
-      <c r="C10" s="89"/>
-      <c r="D10" s="89"/>
-      <c r="E10" s="89"/>
+      <c r="B10" s="79"/>
+      <c r="C10" s="79"/>
+      <c r="D10" s="79"/>
+      <c r="E10" s="79"/>
     </row>
     <row r="11" spans="1:9" ht="15" x14ac:dyDescent="0.25"/>
     <row r="12" spans="1:9" ht="15" x14ac:dyDescent="0.25">
@@ -17234,13 +17234,13 @@
       </c>
     </row>
     <row r="13" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A13" s="87" t="s">
+      <c r="A13" s="77" t="s">
         <v>1070</v>
       </c>
-      <c r="B13" s="87"/>
-      <c r="C13" s="87"/>
-      <c r="D13" s="87"/>
-      <c r="E13" s="87"/>
+      <c r="B13" s="77"/>
+      <c r="C13" s="77"/>
+      <c r="D13" s="77"/>
+      <c r="E13" s="77"/>
     </row>
     <row r="14" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A14" s="52" t="s">
@@ -17311,13 +17311,13 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A18" s="87" t="s">
+      <c r="A18" s="77" t="s">
         <v>1082</v>
       </c>
-      <c r="B18" s="87"/>
-      <c r="C18" s="87"/>
-      <c r="D18" s="87"/>
-      <c r="E18" s="87"/>
+      <c r="B18" s="77"/>
+      <c r="C18" s="77"/>
+      <c r="D18" s="77"/>
+      <c r="E18" s="77"/>
     </row>
     <row r="19" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A19" s="52" t="s">
@@ -17371,13 +17371,13 @@
       </c>
     </row>
     <row r="22" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A22" s="87" t="s">
+      <c r="A22" s="77" t="s">
         <v>1091</v>
       </c>
-      <c r="B22" s="87"/>
-      <c r="C22" s="87"/>
-      <c r="D22" s="87"/>
-      <c r="E22" s="87"/>
+      <c r="B22" s="77"/>
+      <c r="C22" s="77"/>
+      <c r="D22" s="77"/>
+      <c r="E22" s="77"/>
     </row>
     <row r="23" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A23" s="52" t="s">
@@ -17448,13 +17448,13 @@
       </c>
     </row>
     <row r="27" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A27" s="87" t="s">
+      <c r="A27" s="77" t="s">
         <v>1100</v>
       </c>
-      <c r="B27" s="87"/>
-      <c r="C27" s="87"/>
-      <c r="D27" s="87"/>
-      <c r="E27" s="87"/>
+      <c r="B27" s="77"/>
+      <c r="C27" s="77"/>
+      <c r="D27" s="77"/>
+      <c r="E27" s="77"/>
     </row>
     <row r="28" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A28" s="52" t="s">
@@ -17491,13 +17491,13 @@
       </c>
     </row>
     <row r="30" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A30" s="87" t="s">
+      <c r="A30" s="77" t="s">
         <v>1105</v>
       </c>
-      <c r="B30" s="87"/>
-      <c r="C30" s="87"/>
-      <c r="D30" s="87"/>
-      <c r="E30" s="87"/>
+      <c r="B30" s="77"/>
+      <c r="C30" s="77"/>
+      <c r="D30" s="77"/>
+      <c r="E30" s="77"/>
     </row>
     <row r="31" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="52" t="s">
@@ -17670,13 +17670,13 @@
       </c>
     </row>
     <row r="41" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A41" s="87" t="s">
+      <c r="A41" s="77" t="s">
         <v>1134</v>
       </c>
-      <c r="B41" s="87"/>
-      <c r="C41" s="87"/>
-      <c r="D41" s="87"/>
-      <c r="E41" s="87"/>
+      <c r="B41" s="77"/>
+      <c r="C41" s="77"/>
+      <c r="D41" s="77"/>
+      <c r="E41" s="77"/>
     </row>
     <row r="42" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A42" s="52" t="s">
@@ -17764,13 +17764,13 @@
       </c>
     </row>
     <row r="47" spans="1:5" ht="15" x14ac:dyDescent="0.25">
-      <c r="A47" s="87" t="s">
+      <c r="A47" s="77" t="s">
         <v>1135</v>
       </c>
-      <c r="B47" s="87"/>
-      <c r="C47" s="87"/>
-      <c r="D47" s="87"/>
-      <c r="E47" s="87"/>
+      <c r="B47" s="77"/>
+      <c r="C47" s="77"/>
+      <c r="D47" s="77"/>
+      <c r="E47" s="77"/>
     </row>
     <row r="48" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A48" s="52" t="s">
@@ -17879,7 +17879,7 @@
         <v>12.3</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="24" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A58" s="52" t="s">
         <v>1076</v>
       </c>
@@ -17897,7 +17897,7 @@
         <v>98.18</v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="24" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A59" s="52" t="s">
         <v>1078</v>
       </c>
@@ -18419,7 +18419,7 @@
       <c r="D90" s="72"/>
       <c r="E90" s="72"/>
     </row>
-    <row r="91" spans="1:9" ht="24" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A91" s="52" t="s">
         <v>1132</v>
       </c>
@@ -18476,17 +18476,17 @@
     <row r="94" spans="1:9" ht="15" x14ac:dyDescent="0.25"/>
     <row r="95" spans="1:9" ht="15" x14ac:dyDescent="0.25"/>
     <row r="96" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="82" t="s">
+      <c r="A96" s="81" t="s">
         <v>1173</v>
       </c>
-      <c r="B96" s="82"/>
-      <c r="C96" s="82"/>
-      <c r="D96" s="82"/>
-      <c r="E96" s="82"/>
-      <c r="F96" s="82"/>
-      <c r="G96" s="82"/>
-      <c r="H96" s="82"/>
-      <c r="I96" s="82"/>
+      <c r="B96" s="81"/>
+      <c r="C96" s="81"/>
+      <c r="D96" s="81"/>
+      <c r="E96" s="81"/>
+      <c r="F96" s="81"/>
+      <c r="G96" s="81"/>
+      <c r="H96" s="81"/>
+      <c r="I96" s="81"/>
     </row>
     <row r="97" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="59" t="s">
@@ -19458,80 +19458,80 @@
       <c r="I130" s="25"/>
     </row>
     <row r="131" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A131" s="83" t="s">
+      <c r="A131" s="82" t="s">
         <v>1176</v>
       </c>
-      <c r="B131" s="83"/>
-      <c r="C131" s="83"/>
-      <c r="D131" s="83"/>
-      <c r="E131" s="83"/>
-      <c r="F131" s="83"/>
-      <c r="G131" s="83"/>
-      <c r="H131" s="84"/>
-      <c r="I131" s="84"/>
+      <c r="B131" s="82"/>
+      <c r="C131" s="82"/>
+      <c r="D131" s="82"/>
+      <c r="E131" s="82"/>
+      <c r="F131" s="82"/>
+      <c r="G131" s="82"/>
+      <c r="H131" s="83"/>
+      <c r="I131" s="83"/>
     </row>
     <row r="132" spans="1:9" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A132" s="81" t="s">
+      <c r="A132" s="80" t="s">
         <v>1170</v>
       </c>
-      <c r="B132" s="81"/>
+      <c r="B132" s="80"/>
       <c r="C132" s="60">
         <f>SUM(E57:E93)</f>
         <v>710.80000000000007</v>
       </c>
       <c r="D132" s="63"/>
-      <c r="E132" s="85" t="s">
+      <c r="E132" s="84" t="s">
         <v>1212</v>
       </c>
-      <c r="F132" s="85"/>
-      <c r="G132" s="85"/>
-      <c r="H132" s="85"/>
-      <c r="I132" s="85"/>
+      <c r="F132" s="84"/>
+      <c r="G132" s="84"/>
+      <c r="H132" s="84"/>
+      <c r="I132" s="84"/>
     </row>
     <row r="133" spans="1:9" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A133" s="81" t="s">
+      <c r="A133" s="80" t="s">
         <v>1171</v>
       </c>
-      <c r="B133" s="81"/>
+      <c r="B133" s="80"/>
       <c r="C133" s="60">
         <f>C132+(F98-C98)*--D57+(F99-C99)*--D58+(F100-C100)*--D59+(F101-C101)*--D60+(F110-C110)*--D72+(F114-C114)*--D77+(F115-C115)*--D78+(F118-C118)*--D81+(F124-C124)*--D88+(F126-C126)*--D91</f>
         <v>944.54000000000008</v>
       </c>
       <c r="D133" s="63"/>
-      <c r="E133" s="85"/>
-      <c r="F133" s="85"/>
-      <c r="G133" s="85"/>
-      <c r="H133" s="85"/>
-      <c r="I133" s="85"/>
+      <c r="E133" s="84"/>
+      <c r="F133" s="84"/>
+      <c r="G133" s="84"/>
+      <c r="H133" s="84"/>
+      <c r="I133" s="84"/>
     </row>
     <row r="134" spans="1:9" ht="51.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A134" s="81" t="s">
+      <c r="A134" s="80" t="s">
         <v>1172</v>
       </c>
-      <c r="B134" s="81"/>
+      <c r="B134" s="80"/>
       <c r="C134" s="60">
         <f>C133-C132</f>
         <v>233.74</v>
       </c>
       <c r="D134" s="63"/>
-      <c r="E134" s="85"/>
-      <c r="F134" s="85"/>
-      <c r="G134" s="85"/>
-      <c r="H134" s="85"/>
-      <c r="I134" s="85"/>
+      <c r="E134" s="84"/>
+      <c r="F134" s="84"/>
+      <c r="G134" s="84"/>
+      <c r="H134" s="84"/>
+      <c r="I134" s="84"/>
     </row>
     <row r="137" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A137" s="86" t="s">
+      <c r="A137" s="85" t="s">
         <v>1213</v>
       </c>
-      <c r="B137" s="86"/>
-      <c r="C137" s="86"/>
-      <c r="D137" s="86"/>
-      <c r="E137" s="86"/>
-      <c r="F137" s="86"/>
-      <c r="G137" s="86"/>
-      <c r="H137" s="86"/>
-      <c r="I137" s="86"/>
+      <c r="B137" s="85"/>
+      <c r="C137" s="85"/>
+      <c r="D137" s="85"/>
+      <c r="E137" s="85"/>
+      <c r="F137" s="85"/>
+      <c r="G137" s="85"/>
+      <c r="H137" s="85"/>
+      <c r="I137" s="85"/>
     </row>
     <row r="138" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="76"/>
@@ -19545,65 +19545,65 @@
       <c r="I138" s="76"/>
     </row>
     <row r="139" spans="1:9" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A139" s="77" t="s">
+      <c r="A139" s="86" t="s">
         <v>1214</v>
       </c>
-      <c r="B139" s="77"/>
-      <c r="C139" s="77"/>
-      <c r="D139" s="77"/>
-      <c r="E139" s="77"/>
-      <c r="F139" s="77"/>
-      <c r="G139" s="77"/>
-      <c r="H139" s="77"/>
-      <c r="I139" s="77"/>
+      <c r="B139" s="86"/>
+      <c r="C139" s="86"/>
+      <c r="D139" s="86"/>
+      <c r="E139" s="86"/>
+      <c r="F139" s="86"/>
+      <c r="G139" s="86"/>
+      <c r="H139" s="86"/>
+      <c r="I139" s="86"/>
     </row>
     <row r="140" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A140" s="78" t="s">
+      <c r="A140" s="87" t="s">
         <v>1215</v>
       </c>
-      <c r="B140" s="78"/>
-      <c r="C140" s="78"/>
-      <c r="D140" s="78"/>
-      <c r="E140" s="78"/>
-      <c r="F140" s="78"/>
-      <c r="G140" s="78"/>
-      <c r="H140" s="78"/>
-      <c r="I140" s="80" t="s">
+      <c r="B140" s="87"/>
+      <c r="C140" s="87"/>
+      <c r="D140" s="87"/>
+      <c r="E140" s="87"/>
+      <c r="F140" s="87"/>
+      <c r="G140" s="87"/>
+      <c r="H140" s="87"/>
+      <c r="I140" s="89" t="s">
         <v>1216</v>
       </c>
     </row>
     <row r="141" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A141" s="78"/>
-      <c r="B141" s="78"/>
-      <c r="C141" s="78"/>
-      <c r="D141" s="78"/>
-      <c r="E141" s="78"/>
-      <c r="F141" s="78"/>
-      <c r="G141" s="78"/>
-      <c r="H141" s="78"/>
-      <c r="I141" s="80"/>
+      <c r="A141" s="87"/>
+      <c r="B141" s="87"/>
+      <c r="C141" s="87"/>
+      <c r="D141" s="87"/>
+      <c r="E141" s="87"/>
+      <c r="F141" s="87"/>
+      <c r="G141" s="87"/>
+      <c r="H141" s="87"/>
+      <c r="I141" s="89"/>
     </row>
     <row r="142" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A142" s="78"/>
-      <c r="B142" s="78"/>
-      <c r="C142" s="78"/>
-      <c r="D142" s="78"/>
-      <c r="E142" s="78"/>
-      <c r="F142" s="78"/>
-      <c r="G142" s="78"/>
-      <c r="H142" s="78"/>
-      <c r="I142" s="80"/>
+      <c r="A142" s="87"/>
+      <c r="B142" s="87"/>
+      <c r="C142" s="87"/>
+      <c r="D142" s="87"/>
+      <c r="E142" s="87"/>
+      <c r="F142" s="87"/>
+      <c r="G142" s="87"/>
+      <c r="H142" s="87"/>
+      <c r="I142" s="89"/>
     </row>
     <row r="143" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A143" s="79"/>
-      <c r="B143" s="79"/>
-      <c r="C143" s="79"/>
-      <c r="D143" s="79"/>
-      <c r="E143" s="79"/>
-      <c r="F143" s="79"/>
-      <c r="G143" s="79"/>
-      <c r="H143" s="79"/>
-      <c r="I143" s="80"/>
+      <c r="A143" s="88"/>
+      <c r="B143" s="88"/>
+      <c r="C143" s="88"/>
+      <c r="D143" s="88"/>
+      <c r="E143" s="88"/>
+      <c r="F143" s="88"/>
+      <c r="G143" s="88"/>
+      <c r="H143" s="88"/>
+      <c r="I143" s="89"/>
     </row>
     <row r="144" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="76"/>
@@ -19617,54 +19617,54 @@
       <c r="I144" s="76"/>
     </row>
     <row r="145" spans="1:9" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A145" s="77" t="s">
+      <c r="A145" s="86" t="s">
         <v>1217</v>
       </c>
-      <c r="B145" s="77"/>
-      <c r="C145" s="77"/>
-      <c r="D145" s="77"/>
-      <c r="E145" s="77"/>
-      <c r="F145" s="77"/>
-      <c r="G145" s="77"/>
-      <c r="H145" s="77"/>
-      <c r="I145" s="77"/>
+      <c r="B145" s="86"/>
+      <c r="C145" s="86"/>
+      <c r="D145" s="86"/>
+      <c r="E145" s="86"/>
+      <c r="F145" s="86"/>
+      <c r="G145" s="86"/>
+      <c r="H145" s="86"/>
+      <c r="I145" s="86"/>
     </row>
     <row r="146" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A146" s="78" t="s">
+      <c r="A146" s="87" t="s">
         <v>1218</v>
       </c>
-      <c r="B146" s="78"/>
-      <c r="C146" s="78"/>
-      <c r="D146" s="78"/>
-      <c r="E146" s="78"/>
-      <c r="F146" s="78"/>
-      <c r="G146" s="78"/>
-      <c r="H146" s="78"/>
-      <c r="I146" s="80" t="s">
+      <c r="B146" s="87"/>
+      <c r="C146" s="87"/>
+      <c r="D146" s="87"/>
+      <c r="E146" s="87"/>
+      <c r="F146" s="87"/>
+      <c r="G146" s="87"/>
+      <c r="H146" s="87"/>
+      <c r="I146" s="89" t="s">
         <v>1219</v>
       </c>
     </row>
     <row r="147" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A147" s="78"/>
-      <c r="B147" s="78"/>
-      <c r="C147" s="78"/>
-      <c r="D147" s="78"/>
-      <c r="E147" s="78"/>
-      <c r="F147" s="78"/>
-      <c r="G147" s="78"/>
-      <c r="H147" s="78"/>
-      <c r="I147" s="80"/>
+      <c r="A147" s="87"/>
+      <c r="B147" s="87"/>
+      <c r="C147" s="87"/>
+      <c r="D147" s="87"/>
+      <c r="E147" s="87"/>
+      <c r="F147" s="87"/>
+      <c r="G147" s="87"/>
+      <c r="H147" s="87"/>
+      <c r="I147" s="89"/>
     </row>
     <row r="148" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A148" s="79"/>
-      <c r="B148" s="79"/>
-      <c r="C148" s="79"/>
-      <c r="D148" s="79"/>
-      <c r="E148" s="79"/>
-      <c r="F148" s="79"/>
-      <c r="G148" s="79"/>
-      <c r="H148" s="79"/>
-      <c r="I148" s="80"/>
+      <c r="A148" s="88"/>
+      <c r="B148" s="88"/>
+      <c r="C148" s="88"/>
+      <c r="D148" s="88"/>
+      <c r="E148" s="88"/>
+      <c r="F148" s="88"/>
+      <c r="G148" s="88"/>
+      <c r="H148" s="88"/>
+      <c r="I148" s="89"/>
     </row>
     <row r="149" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="76"/>
@@ -19678,68 +19678,84 @@
       <c r="I149" s="76"/>
     </row>
     <row r="150" spans="1:9" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A150" s="77" t="s">
+      <c r="A150" s="86" t="s">
         <v>1220</v>
       </c>
-      <c r="B150" s="77"/>
-      <c r="C150" s="77"/>
-      <c r="D150" s="77"/>
-      <c r="E150" s="77"/>
-      <c r="F150" s="77"/>
-      <c r="G150" s="77"/>
-      <c r="H150" s="77"/>
-      <c r="I150" s="77"/>
+      <c r="B150" s="86"/>
+      <c r="C150" s="86"/>
+      <c r="D150" s="86"/>
+      <c r="E150" s="86"/>
+      <c r="F150" s="86"/>
+      <c r="G150" s="86"/>
+      <c r="H150" s="86"/>
+      <c r="I150" s="86"/>
     </row>
     <row r="151" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A151" s="78" t="s">
+      <c r="A151" s="87" t="s">
         <v>1221</v>
       </c>
-      <c r="B151" s="78"/>
-      <c r="C151" s="78"/>
-      <c r="D151" s="78"/>
-      <c r="E151" s="78"/>
-      <c r="F151" s="78"/>
-      <c r="G151" s="78"/>
-      <c r="H151" s="78"/>
-      <c r="I151" s="80" t="s">
+      <c r="B151" s="87"/>
+      <c r="C151" s="87"/>
+      <c r="D151" s="87"/>
+      <c r="E151" s="87"/>
+      <c r="F151" s="87"/>
+      <c r="G151" s="87"/>
+      <c r="H151" s="87"/>
+      <c r="I151" s="89" t="s">
         <v>1222</v>
       </c>
     </row>
     <row r="152" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A152" s="78"/>
-      <c r="B152" s="78"/>
-      <c r="C152" s="78"/>
-      <c r="D152" s="78"/>
-      <c r="E152" s="78"/>
-      <c r="F152" s="78"/>
-      <c r="G152" s="78"/>
-      <c r="H152" s="78"/>
-      <c r="I152" s="80"/>
+      <c r="A152" s="87"/>
+      <c r="B152" s="87"/>
+      <c r="C152" s="87"/>
+      <c r="D152" s="87"/>
+      <c r="E152" s="87"/>
+      <c r="F152" s="87"/>
+      <c r="G152" s="87"/>
+      <c r="H152" s="87"/>
+      <c r="I152" s="89"/>
     </row>
     <row r="153" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A153" s="78"/>
-      <c r="B153" s="78"/>
-      <c r="C153" s="78"/>
-      <c r="D153" s="78"/>
-      <c r="E153" s="78"/>
-      <c r="F153" s="78"/>
-      <c r="G153" s="78"/>
-      <c r="H153" s="78"/>
-      <c r="I153" s="80"/>
+      <c r="A153" s="87"/>
+      <c r="B153" s="87"/>
+      <c r="C153" s="87"/>
+      <c r="D153" s="87"/>
+      <c r="E153" s="87"/>
+      <c r="F153" s="87"/>
+      <c r="G153" s="87"/>
+      <c r="H153" s="87"/>
+      <c r="I153" s="89"/>
     </row>
     <row r="154" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A154" s="79"/>
-      <c r="B154" s="79"/>
-      <c r="C154" s="79"/>
-      <c r="D154" s="79"/>
-      <c r="E154" s="79"/>
-      <c r="F154" s="79"/>
-      <c r="G154" s="79"/>
-      <c r="H154" s="79"/>
-      <c r="I154" s="80"/>
+      <c r="A154" s="88"/>
+      <c r="B154" s="88"/>
+      <c r="C154" s="88"/>
+      <c r="D154" s="88"/>
+      <c r="E154" s="88"/>
+      <c r="F154" s="88"/>
+      <c r="G154" s="88"/>
+      <c r="H154" s="88"/>
+      <c r="I154" s="89"/>
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="A150:I150"/>
+    <mergeCell ref="A151:H154"/>
+    <mergeCell ref="I151:I154"/>
+    <mergeCell ref="A139:I139"/>
+    <mergeCell ref="A140:H143"/>
+    <mergeCell ref="I140:I143"/>
+    <mergeCell ref="A145:I145"/>
+    <mergeCell ref="A146:H148"/>
+    <mergeCell ref="I146:I148"/>
+    <mergeCell ref="A134:B134"/>
+    <mergeCell ref="A96:I96"/>
+    <mergeCell ref="A131:I131"/>
+    <mergeCell ref="E132:I134"/>
+    <mergeCell ref="A137:I137"/>
+    <mergeCell ref="A132:B132"/>
+    <mergeCell ref="A133:B133"/>
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="A41:E41"/>
     <mergeCell ref="A47:E47"/>
@@ -19749,22 +19765,6 @@
     <mergeCell ref="A18:E18"/>
     <mergeCell ref="A22:E22"/>
     <mergeCell ref="A27:E27"/>
-    <mergeCell ref="A134:B134"/>
-    <mergeCell ref="A96:I96"/>
-    <mergeCell ref="A131:I131"/>
-    <mergeCell ref="E132:I134"/>
-    <mergeCell ref="A137:I137"/>
-    <mergeCell ref="A132:B132"/>
-    <mergeCell ref="A133:B133"/>
-    <mergeCell ref="A150:I150"/>
-    <mergeCell ref="A151:H154"/>
-    <mergeCell ref="I151:I154"/>
-    <mergeCell ref="A139:I139"/>
-    <mergeCell ref="A140:H143"/>
-    <mergeCell ref="I140:I143"/>
-    <mergeCell ref="A145:I145"/>
-    <mergeCell ref="A146:H148"/>
-    <mergeCell ref="I146:I148"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="I101" r:id="rId1" xr:uid="{005B6573-1B63-4272-AEDD-EACA4DDEA04C}"/>

</xml_diff>